<commit_message>
Classifier stage 2 and Classifier 3 classes
Since stage 2 classifier for clustered and unclustered has a high accuracy off the bat 93%, I want to check if having a 3 stage classifier with Nonmono, clustered and unclustered yields a higher cumulative accuracy.
</commit_message>
<xml_diff>
--- a/experiment_log.xlsx
+++ b/experiment_log.xlsx
@@ -510,7 +510,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AO15"/>
+  <dimension ref="A1:AO27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2411,7 +2411,6 @@
           <t>2026-03-09</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
           <t>ResNet34</t>
@@ -2535,6 +2534,1659 @@
       </c>
       <c r="AM15" t="n">
         <v>0.7397</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>14</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>ResNet34</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>ImageNet</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H16" t="n">
+        <v>12494</v>
+      </c>
+      <c r="I16" t="n">
+        <v>70</v>
+      </c>
+      <c r="J16" t="n">
+        <v>10</v>
+      </c>
+      <c r="K16" t="n">
+        <v>20</v>
+      </c>
+      <c r="L16" t="n">
+        <v>2211</v>
+      </c>
+      <c r="M16" t="n">
+        <v>2211</v>
+      </c>
+      <c r="N16" t="n">
+        <v>737</v>
+      </c>
+      <c r="O16" t="n">
+        <v>737</v>
+      </c>
+      <c r="P16" t="n">
+        <v>737</v>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>Fixed [1.0, 3.0]</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>AdamW</t>
+        </is>
+      </c>
+      <c r="S16" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="T16" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="U16" t="n">
+        <v>32</v>
+      </c>
+      <c r="V16" t="n">
+        <v>50</v>
+      </c>
+      <c r="W16" t="inlineStr">
+        <is>
+          <t>ReduceLROnPlateau(factor=0.5, patience=3)</t>
+        </is>
+      </c>
+      <c r="X16" t="inlineStr">
+        <is>
+          <t>256x256</t>
+        </is>
+      </c>
+      <c r="Y16" t="inlineStr">
+        <is>
+          <t>HFlip, VFlip, Rot(15°), ColorJitter(b=0.3,c=0.3,s=0.2,h=0.05), Grayscale(0.05), GaussianBlur, Affine(t=0.05)</t>
+        </is>
+      </c>
+      <c r="Z16" t="n">
+        <v>0.9072</v>
+      </c>
+      <c r="AA16" t="n">
+        <v>0.9345</v>
+      </c>
+      <c r="AB16" t="n">
+        <v>0.5395</v>
+      </c>
+      <c r="AC16" t="n">
+        <v>0.6841</v>
+      </c>
+      <c r="AD16" t="n">
+        <v>0.9039</v>
+      </c>
+      <c r="AE16" t="n">
+        <v>0.9913</v>
+      </c>
+      <c r="AF16" t="n">
+        <v>0.9456</v>
+      </c>
+      <c r="AG16" t="n">
+        <v>0.8148</v>
+      </c>
+      <c r="AH16" t="n">
+        <v>0.8969</v>
+      </c>
+      <c r="AI16" t="n">
+        <v>2520</v>
+      </c>
+      <c r="AJ16" t="n">
+        <v>314</v>
+      </c>
+      <c r="AK16" t="n">
+        <v>268</v>
+      </c>
+      <c r="AL16" t="n">
+        <v>22</v>
+      </c>
+      <c r="AM16" t="n">
+        <v>0.9026</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>15</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2026-03-10</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>ResNet34</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>ImageNet</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H17" t="n">
+        <v>12494</v>
+      </c>
+      <c r="I17" t="n">
+        <v>70</v>
+      </c>
+      <c r="J17" t="n">
+        <v>10</v>
+      </c>
+      <c r="K17" t="n">
+        <v>20</v>
+      </c>
+      <c r="L17" t="n">
+        <v>2211</v>
+      </c>
+      <c r="M17" t="n">
+        <v>2211</v>
+      </c>
+      <c r="N17" t="n">
+        <v>737</v>
+      </c>
+      <c r="O17" t="n">
+        <v>737</v>
+      </c>
+      <c r="P17" t="n">
+        <v>737</v>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>Fixed [1.0, 1.5]</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>AdamW</t>
+        </is>
+      </c>
+      <c r="S17" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="T17" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="U17" t="n">
+        <v>32</v>
+      </c>
+      <c r="V17" t="n">
+        <v>50</v>
+      </c>
+      <c r="W17" t="inlineStr">
+        <is>
+          <t>ReduceLROnPlateau(factor=0.5, patience=3)</t>
+        </is>
+      </c>
+      <c r="X17" t="inlineStr">
+        <is>
+          <t>256x256</t>
+        </is>
+      </c>
+      <c r="Y17" t="inlineStr">
+        <is>
+          <t>HFlip, VFlip, Rot(15°), ColorJitter(b=0.3,c=0.3,s=0.2,h=0.05), Grayscale(0.05), GaussianBlur, Affine(t=0.05)</t>
+        </is>
+      </c>
+      <c r="Z17" t="n">
+        <v>0.9069</v>
+      </c>
+      <c r="AA17" t="n">
+        <v>0.9145</v>
+      </c>
+      <c r="AB17" t="n">
+        <v>0.5515</v>
+      </c>
+      <c r="AC17" t="n">
+        <v>0.6881</v>
+      </c>
+      <c r="AD17" t="n">
+        <v>0.9059</v>
+      </c>
+      <c r="AE17" t="n">
+        <v>0.9882</v>
+      </c>
+      <c r="AF17" t="n">
+        <v>0.9452</v>
+      </c>
+      <c r="AG17" t="n">
+        <v>0.8167</v>
+      </c>
+      <c r="AH17" t="n">
+        <v>0.8973</v>
+      </c>
+      <c r="AI17" t="n">
+        <v>2512</v>
+      </c>
+      <c r="AJ17" t="n">
+        <v>321</v>
+      </c>
+      <c r="AK17" t="n">
+        <v>261</v>
+      </c>
+      <c r="AL17" t="n">
+        <v>30</v>
+      </c>
+      <c r="AM17" t="n">
+        <v>0.9083</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>16</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2026-03-10</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>ResNet34</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>ImageNet</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H18" t="n">
+        <v>12494</v>
+      </c>
+      <c r="I18" t="n">
+        <v>70</v>
+      </c>
+      <c r="J18" t="n">
+        <v>10</v>
+      </c>
+      <c r="K18" t="n">
+        <v>20</v>
+      </c>
+      <c r="L18" t="n">
+        <v>2211</v>
+      </c>
+      <c r="M18" t="n">
+        <v>2211</v>
+      </c>
+      <c r="N18" t="n">
+        <v>737</v>
+      </c>
+      <c r="O18" t="n">
+        <v>737</v>
+      </c>
+      <c r="P18" t="n">
+        <v>737</v>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>Fixed [1.0, 1.0]</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>AdamW</t>
+        </is>
+      </c>
+      <c r="S18" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="T18" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="U18" t="n">
+        <v>32</v>
+      </c>
+      <c r="V18" t="n">
+        <v>50</v>
+      </c>
+      <c r="W18" t="inlineStr">
+        <is>
+          <t>ReduceLROnPlateau(factor=0.5, patience=3)</t>
+        </is>
+      </c>
+      <c r="X18" t="inlineStr">
+        <is>
+          <t>256x256</t>
+        </is>
+      </c>
+      <c r="Y18" t="inlineStr">
+        <is>
+          <t>HFlip, VFlip, Rot(15°), ColorJitter(b=0.3,c=0.3,s=0.2,h=0.05), Grayscale(0.05), GaussianBlur, Affine(t=0.05)</t>
+        </is>
+      </c>
+      <c r="Z18" t="n">
+        <v>0.9101</v>
+      </c>
+      <c r="AA18" t="n">
+        <v>0.8698</v>
+      </c>
+      <c r="AB18" t="n">
+        <v>0.6082</v>
+      </c>
+      <c r="AC18" t="n">
+        <v>0.7159</v>
+      </c>
+      <c r="AD18" t="n">
+        <v>0.9161</v>
+      </c>
+      <c r="AE18" t="n">
+        <v>0.9792</v>
+      </c>
+      <c r="AF18" t="n">
+        <v>0.9466</v>
+      </c>
+      <c r="AG18" t="n">
+        <v>0.8312</v>
+      </c>
+      <c r="AH18" t="n">
+        <v>0.9036</v>
+      </c>
+      <c r="AI18" t="n">
+        <v>2489</v>
+      </c>
+      <c r="AJ18" t="n">
+        <v>354</v>
+      </c>
+      <c r="AK18" t="n">
+        <v>228</v>
+      </c>
+      <c r="AL18" t="n">
+        <v>53</v>
+      </c>
+      <c r="AM18" t="n">
+        <v>0.9071</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>17</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2026-03-10</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>ResNet34</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>ImageNet</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G19" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H19" t="n">
+        <v>12494</v>
+      </c>
+      <c r="I19" t="n">
+        <v>70</v>
+      </c>
+      <c r="J19" t="n">
+        <v>10</v>
+      </c>
+      <c r="K19" t="n">
+        <v>20</v>
+      </c>
+      <c r="L19" t="n">
+        <v>2211</v>
+      </c>
+      <c r="M19" t="n">
+        <v>2211</v>
+      </c>
+      <c r="N19" t="n">
+        <v>737</v>
+      </c>
+      <c r="O19" t="n">
+        <v>737</v>
+      </c>
+      <c r="P19" t="n">
+        <v>737</v>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>Inverse natural frequency</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>AdamW</t>
+        </is>
+      </c>
+      <c r="S19" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="T19" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="U19" t="n">
+        <v>32</v>
+      </c>
+      <c r="V19" t="n">
+        <v>20</v>
+      </c>
+      <c r="W19" t="inlineStr">
+        <is>
+          <t>CosineAnnealingLR (T_max=20)</t>
+        </is>
+      </c>
+      <c r="X19" t="inlineStr">
+        <is>
+          <t>256x256</t>
+        </is>
+      </c>
+      <c r="Y19" t="inlineStr">
+        <is>
+          <t>HFlip, VFlip, Rotation(15°), ColorJitter(b=0.2,c=0.2), ImageNet norm</t>
+        </is>
+      </c>
+      <c r="Z19" t="n">
+        <v>0.8147</v>
+      </c>
+      <c r="AA19" t="n">
+        <v>0.5014</v>
+      </c>
+      <c r="AB19" t="n">
+        <v>0.9157999999999999</v>
+      </c>
+      <c r="AC19" t="n">
+        <v>0.648</v>
+      </c>
+      <c r="AD19" t="n">
+        <v>0.9762</v>
+      </c>
+      <c r="AE19" t="n">
+        <v>0.7915</v>
+      </c>
+      <c r="AF19" t="n">
+        <v>0.8742</v>
+      </c>
+      <c r="AG19" t="n">
+        <v>0.7611</v>
+      </c>
+      <c r="AH19" t="n">
+        <v>0.8321</v>
+      </c>
+      <c r="AI19" t="n">
+        <v>2012</v>
+      </c>
+      <c r="AJ19" t="n">
+        <v>533</v>
+      </c>
+      <c r="AK19" t="n">
+        <v>49</v>
+      </c>
+      <c r="AL19" t="n">
+        <v>530</v>
+      </c>
+      <c r="AM19" t="n">
+        <v>0.8071</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>18</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2026-03-10</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>4-class training collapsed to binary — NonMono subclass split</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>ResNet34</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>ImageNet</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G20" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H20" t="n">
+        <v>12494</v>
+      </c>
+      <c r="I20" t="n">
+        <v>70</v>
+      </c>
+      <c r="J20" t="n">
+        <v>10</v>
+      </c>
+      <c r="K20" t="n">
+        <v>20</v>
+      </c>
+      <c r="L20" t="n">
+        <v>1200</v>
+      </c>
+      <c r="M20" t="n">
+        <v>1500</v>
+      </c>
+      <c r="N20" t="n">
+        <v>500</v>
+      </c>
+      <c r="O20" t="n">
+        <v>500</v>
+      </c>
+      <c r="P20" t="n">
+        <v>500</v>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>Inverse natural frequency (per subclass)</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>AdamW</t>
+        </is>
+      </c>
+      <c r="S20" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="T20" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="U20" t="n">
+        <v>32</v>
+      </c>
+      <c r="V20" t="n">
+        <v>20</v>
+      </c>
+      <c r="W20" t="inlineStr">
+        <is>
+          <t>CosineAnnealingLR (T_max=20)</t>
+        </is>
+      </c>
+      <c r="X20" t="inlineStr">
+        <is>
+          <t>256x256</t>
+        </is>
+      </c>
+      <c r="Y20" t="inlineStr">
+        <is>
+          <t>HFlip, VFlip, Rotation(15°), ColorJitter(b=0.2,c=0.2), ImageNet norm</t>
+        </is>
+      </c>
+      <c r="Z20" t="n">
+        <v>0.8784</v>
+      </c>
+      <c r="AA20" t="n">
+        <v>0.6332</v>
+      </c>
+      <c r="AB20" t="n">
+        <v>0.8247</v>
+      </c>
+      <c r="AC20" t="n">
+        <v>0.7164</v>
+      </c>
+      <c r="AD20" t="n">
+        <v>0.9569</v>
+      </c>
+      <c r="AE20" t="n">
+        <v>0.8905999999999999</v>
+      </c>
+      <c r="AF20" t="n">
+        <v>0.9226</v>
+      </c>
+      <c r="AG20" t="n">
+        <v>0.8195</v>
+      </c>
+      <c r="AH20" t="n">
+        <v>0.8842</v>
+      </c>
+      <c r="AI20" t="n">
+        <v>2264</v>
+      </c>
+      <c r="AJ20" t="n">
+        <v>480</v>
+      </c>
+      <c r="AK20" t="n">
+        <v>102</v>
+      </c>
+      <c r="AL20" t="n">
+        <v>278</v>
+      </c>
+      <c r="AM20" t="n">
+        <v>0.8846000000000001</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>19</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>2026-03-10</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>3-class training: Unusable+Lymphocyte / RBCalone / Monocyte — collapsed to binary</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>ResNet34</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>ImageNet</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G21" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H21" t="n">
+        <v>12494</v>
+      </c>
+      <c r="I21" t="n">
+        <v>70</v>
+      </c>
+      <c r="J21" t="n">
+        <v>10</v>
+      </c>
+      <c r="K21" t="n">
+        <v>20</v>
+      </c>
+      <c r="L21" t="n">
+        <v>1200</v>
+      </c>
+      <c r="M21" t="n">
+        <v>2211</v>
+      </c>
+      <c r="N21" t="n">
+        <v>737</v>
+      </c>
+      <c r="O21" t="n">
+        <v>737</v>
+      </c>
+      <c r="P21" t="n">
+        <v>737</v>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>Per-subclass inverse frequency (3-class training)</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>AdamW</t>
+        </is>
+      </c>
+      <c r="S21" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="T21" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="U21" t="n">
+        <v>32</v>
+      </c>
+      <c r="V21" t="n">
+        <v>20</v>
+      </c>
+      <c r="W21" t="inlineStr">
+        <is>
+          <t>CosineAnnealingLR (T_max=20)</t>
+        </is>
+      </c>
+      <c r="X21" t="inlineStr">
+        <is>
+          <t>256x256</t>
+        </is>
+      </c>
+      <c r="Y21" t="inlineStr">
+        <is>
+          <t>HFlip, VFlip, Rotation(15°), ColorJitter(b=0.2,c=0.2), ImageNet norm</t>
+        </is>
+      </c>
+      <c r="Z21" t="n">
+        <v>0.9165</v>
+      </c>
+      <c r="AA21" t="n">
+        <v>0.7801</v>
+      </c>
+      <c r="AB21" t="n">
+        <v>0.768</v>
+      </c>
+      <c r="AC21" t="n">
+        <v>0.774</v>
+      </c>
+      <c r="AD21" t="n">
+        <v>0.9471000000000001</v>
+      </c>
+      <c r="AE21" t="n">
+        <v>0.9504</v>
+      </c>
+      <c r="AF21" t="n">
+        <v>0.9488</v>
+      </c>
+      <c r="AG21" t="n">
+        <v>0.8614000000000001</v>
+      </c>
+      <c r="AH21" t="n">
+        <v>0.9162</v>
+      </c>
+      <c r="AI21" t="n">
+        <v>2416</v>
+      </c>
+      <c r="AJ21" t="n">
+        <v>447</v>
+      </c>
+      <c r="AK21" t="n">
+        <v>135</v>
+      </c>
+      <c r="AL21" t="n">
+        <v>126</v>
+      </c>
+      <c r="AM21" t="n">
+        <v>0.9051</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>20</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2026-03-11</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>3-class training: Unusable+Lymphocyte / RBCalone / Monocyte — collapsed to binary</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>ResNet34</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>ImageNet</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G22" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H22" t="n">
+        <v>12494</v>
+      </c>
+      <c r="I22" t="n">
+        <v>70</v>
+      </c>
+      <c r="J22" t="n">
+        <v>10</v>
+      </c>
+      <c r="K22" t="n">
+        <v>20</v>
+      </c>
+      <c r="L22" t="n">
+        <v>1200</v>
+      </c>
+      <c r="M22" t="n">
+        <v>2211</v>
+      </c>
+      <c r="N22" t="n">
+        <v>737</v>
+      </c>
+      <c r="O22" t="n">
+        <v>737</v>
+      </c>
+      <c r="P22" t="n">
+        <v>737</v>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>Per-subclass inverse frequency (3-class training)</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>AdamW</t>
+        </is>
+      </c>
+      <c r="S22" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="T22" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="U22" t="n">
+        <v>32</v>
+      </c>
+      <c r="V22" t="n">
+        <v>20</v>
+      </c>
+      <c r="W22" t="inlineStr">
+        <is>
+          <t>CosineAnnealingLR (T_max=20)</t>
+        </is>
+      </c>
+      <c r="X22" t="inlineStr">
+        <is>
+          <t>256x256</t>
+        </is>
+      </c>
+      <c r="Y22" t="inlineStr">
+        <is>
+          <t>HFlip, VFlip, Rotation(15°), ColorJitter(b=0.2,c=0.2), ImageNet norm</t>
+        </is>
+      </c>
+      <c r="Z22" t="n">
+        <v>0.8848</v>
+      </c>
+      <c r="AA22" t="n">
+        <v>0.6581</v>
+      </c>
+      <c r="AB22" t="n">
+        <v>0.7938</v>
+      </c>
+      <c r="AC22" t="n">
+        <v>0.7196</v>
+      </c>
+      <c r="AD22" t="n">
+        <v>0.9505</v>
+      </c>
+      <c r="AE22" t="n">
+        <v>0.9056</v>
+      </c>
+      <c r="AF22" t="n">
+        <v>0.9275</v>
+      </c>
+      <c r="AG22" t="n">
+        <v>0.8236</v>
+      </c>
+      <c r="AH22" t="n">
+        <v>0.8888</v>
+      </c>
+      <c r="AI22" t="n">
+        <v>2302</v>
+      </c>
+      <c r="AJ22" t="n">
+        <v>462</v>
+      </c>
+      <c r="AK22" t="n">
+        <v>120</v>
+      </c>
+      <c r="AL22" t="n">
+        <v>240</v>
+      </c>
+      <c r="AM22" t="n">
+        <v>0.884</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>21</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>2026-03-11</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>3-class training: Unusable+Lymphocyte / RBCalone / Monocyte — collapsed to binary</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>ResNet34</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>ImageNet</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G23" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H23" t="n">
+        <v>12494</v>
+      </c>
+      <c r="I23" t="n">
+        <v>70</v>
+      </c>
+      <c r="J23" t="n">
+        <v>10</v>
+      </c>
+      <c r="K23" t="n">
+        <v>20</v>
+      </c>
+      <c r="L23" t="n">
+        <v>1200</v>
+      </c>
+      <c r="M23" t="n">
+        <v>2211</v>
+      </c>
+      <c r="N23" t="n">
+        <v>737</v>
+      </c>
+      <c r="O23" t="n">
+        <v>737</v>
+      </c>
+      <c r="P23" t="n">
+        <v>737</v>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>Per-subclass inverse frequency (3-class training)</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>AdamW</t>
+        </is>
+      </c>
+      <c r="S23" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="T23" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="U23" t="n">
+        <v>32</v>
+      </c>
+      <c r="V23" t="n">
+        <v>20</v>
+      </c>
+      <c r="W23" t="inlineStr">
+        <is>
+          <t>CosineAnnealingLR (T_max=20)</t>
+        </is>
+      </c>
+      <c r="X23" t="inlineStr">
+        <is>
+          <t>256x256</t>
+        </is>
+      </c>
+      <c r="Y23" t="inlineStr">
+        <is>
+          <t>HFlip, VFlip, Rotation(15°), ColorJitter(b=0.2,c=0.2), ImageNet norm</t>
+        </is>
+      </c>
+      <c r="Z23" t="n">
+        <v>0.8921</v>
+      </c>
+      <c r="AA23" t="n">
+        <v>0.6783</v>
+      </c>
+      <c r="AB23" t="n">
+        <v>0.8007</v>
+      </c>
+      <c r="AC23" t="n">
+        <v>0.7344000000000001</v>
+      </c>
+      <c r="AD23" t="n">
+        <v>0.9524</v>
+      </c>
+      <c r="AE23" t="n">
+        <v>0.9131</v>
+      </c>
+      <c r="AF23" t="n">
+        <v>0.9323</v>
+      </c>
+      <c r="AG23" t="n">
+        <v>0.8334</v>
+      </c>
+      <c r="AH23" t="n">
+        <v>0.8955</v>
+      </c>
+      <c r="AI23" t="n">
+        <v>2321</v>
+      </c>
+      <c r="AJ23" t="n">
+        <v>466</v>
+      </c>
+      <c r="AK23" t="n">
+        <v>116</v>
+      </c>
+      <c r="AL23" t="n">
+        <v>221</v>
+      </c>
+      <c r="AM23" t="n">
+        <v>0.8872</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>22</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>2026-03-11</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Stage2 — 2-class clean</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>ResNet34</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>ImageNet</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G24" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Stage2</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>70</v>
+      </c>
+      <c r="J24" t="n">
+        <v>10</v>
+      </c>
+      <c r="K24" t="n">
+        <v>20</v>
+      </c>
+      <c r="L24" t="n">
+        <v>1800</v>
+      </c>
+      <c r="M24" t="n">
+        <v>1800</v>
+      </c>
+      <c r="N24" t="n">
+        <v>900</v>
+      </c>
+      <c r="O24" t="n">
+        <v>900</v>
+      </c>
+      <c r="P24" t="n">
+        <v>1800</v>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>Equal balance per subclass — mode: 2-class clean</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>AdamW</t>
+        </is>
+      </c>
+      <c r="S24" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="T24" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="U24" t="n">
+        <v>32</v>
+      </c>
+      <c r="V24" t="n">
+        <v>20</v>
+      </c>
+      <c r="W24" t="inlineStr">
+        <is>
+          <t>CosineAnnealingLR (T_max=20)</t>
+        </is>
+      </c>
+      <c r="X24" t="inlineStr">
+        <is>
+          <t>256x256</t>
+        </is>
+      </c>
+      <c r="Y24" t="inlineStr">
+        <is>
+          <t>HFlip, VFlip, Rotation(15°), ColorJitter(b=0.2,c=0.2), ImageNet norm</t>
+        </is>
+      </c>
+      <c r="Z24" t="n">
+        <v>0.9252</v>
+      </c>
+      <c r="AA24" t="n">
+        <v>0.8919</v>
+      </c>
+      <c r="AB24" t="n">
+        <v>0.9574</v>
+      </c>
+      <c r="AC24" t="n">
+        <v>0.9235</v>
+      </c>
+      <c r="AD24" t="n">
+        <v>0.9594</v>
+      </c>
+      <c r="AE24" t="n">
+        <v>0.8965</v>
+      </c>
+      <c r="AF24" t="n">
+        <v>0.9268999999999999</v>
+      </c>
+      <c r="AG24" t="n">
+        <v>0.9252</v>
+      </c>
+      <c r="AH24" t="n">
+        <v>0.9253</v>
+      </c>
+      <c r="AI24" t="n">
+        <v>1204</v>
+      </c>
+      <c r="AJ24" t="n">
+        <v>1147</v>
+      </c>
+      <c r="AK24" t="n">
+        <v>51</v>
+      </c>
+      <c r="AL24" t="n">
+        <v>139</v>
+      </c>
+      <c r="AM24" t="n">
+        <v>0.9323</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>23</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>2026-03-11</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Stage2 — 3-class+reject</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>ResNet34</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>ImageNet</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G25" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Stage2</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
+        <v>70</v>
+      </c>
+      <c r="J25" t="n">
+        <v>10</v>
+      </c>
+      <c r="K25" t="n">
+        <v>20</v>
+      </c>
+      <c r="L25" t="n">
+        <v>1800</v>
+      </c>
+      <c r="M25" t="n">
+        <v>1800</v>
+      </c>
+      <c r="N25" t="n">
+        <v>900</v>
+      </c>
+      <c r="O25" t="n">
+        <v>900</v>
+      </c>
+      <c r="P25" t="n">
+        <v>1800</v>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>Equal balance per subclass — mode: 3-class+reject</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>AdamW</t>
+        </is>
+      </c>
+      <c r="S25" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="T25" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="U25" t="n">
+        <v>32</v>
+      </c>
+      <c r="V25" t="n">
+        <v>20</v>
+      </c>
+      <c r="W25" t="inlineStr">
+        <is>
+          <t>CosineAnnealingLR (T_max=20)</t>
+        </is>
+      </c>
+      <c r="X25" t="inlineStr">
+        <is>
+          <t>256x256</t>
+        </is>
+      </c>
+      <c r="Y25" t="inlineStr">
+        <is>
+          <t>HFlip, VFlip, Rotation(15°), ColorJitter(b=0.2,c=0.2), ImageNet norm</t>
+        </is>
+      </c>
+      <c r="Z25" t="n">
+        <v>0.9197</v>
+      </c>
+      <c r="AA25" t="n">
+        <v>0.8981</v>
+      </c>
+      <c r="AB25" t="n">
+        <v>0.9558</v>
+      </c>
+      <c r="AC25" t="n">
+        <v>0.9261</v>
+      </c>
+      <c r="AD25" t="n">
+        <v>0.9605</v>
+      </c>
+      <c r="AE25" t="n">
+        <v>0.8875999999999999</v>
+      </c>
+      <c r="AF25" t="n">
+        <v>0.9226</v>
+      </c>
+      <c r="AG25" t="n">
+        <v>0.9243</v>
+      </c>
+      <c r="AH25" t="n">
+        <v>0.9242</v>
+      </c>
+      <c r="AI25" t="n">
+        <v>1192</v>
+      </c>
+      <c r="AJ25" t="n">
+        <v>1146</v>
+      </c>
+      <c r="AK25" t="n">
+        <v>49</v>
+      </c>
+      <c r="AL25" t="n">
+        <v>130</v>
+      </c>
+      <c r="AM25" t="n">
+        <v>0.9228</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>24</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>2026-03-11</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Stage 2 — Clustered vs Unclustered</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>ResNet34</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>ImageNet</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G26" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Stage2</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>70</v>
+      </c>
+      <c r="J26" t="n">
+        <v>10</v>
+      </c>
+      <c r="K26" t="n">
+        <v>20</v>
+      </c>
+      <c r="L26" t="n">
+        <v>1800</v>
+      </c>
+      <c r="M26" t="n">
+        <v>1800</v>
+      </c>
+      <c r="N26" t="n">
+        <v>900</v>
+      </c>
+      <c r="O26" t="n">
+        <v>900</v>
+      </c>
+      <c r="P26" t="n">
+        <v>1800</v>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>Equal balance per subclass</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>AdamW</t>
+        </is>
+      </c>
+      <c r="S26" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="T26" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="U26" t="n">
+        <v>32</v>
+      </c>
+      <c r="V26" t="n">
+        <v>30</v>
+      </c>
+      <c r="W26" t="inlineStr">
+        <is>
+          <t>CosineAnnealingLR (T_max=30)</t>
+        </is>
+      </c>
+      <c r="X26" t="inlineStr">
+        <is>
+          <t>256x256</t>
+        </is>
+      </c>
+      <c r="Y26" t="inlineStr">
+        <is>
+          <t>HFlip, VFlip, Rotation(15°), ColorJitter(b=0.2,c=0.2), ImageNet norm</t>
+        </is>
+      </c>
+      <c r="Z26" t="n">
+        <v>0.9256</v>
+      </c>
+      <c r="AA26" t="n">
+        <v>0.902</v>
+      </c>
+      <c r="AB26" t="n">
+        <v>0.9449</v>
+      </c>
+      <c r="AC26" t="n">
+        <v>0.923</v>
+      </c>
+      <c r="AD26" t="n">
+        <v>0.9487</v>
+      </c>
+      <c r="AE26" t="n">
+        <v>0.9084</v>
+      </c>
+      <c r="AF26" t="n">
+        <v>0.9281</v>
+      </c>
+      <c r="AG26" t="n">
+        <v>0.9255</v>
+      </c>
+      <c r="AH26" t="n">
+        <v>0.9257</v>
+      </c>
+      <c r="AI26" t="n">
+        <v>1220</v>
+      </c>
+      <c r="AJ26" t="n">
+        <v>1132</v>
+      </c>
+      <c r="AK26" t="n">
+        <v>66</v>
+      </c>
+      <c r="AL26" t="n">
+        <v>123</v>
+      </c>
+      <c r="AM26" t="n">
+        <v>0.9307</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>25</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>2026-03-11</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>3-class single model — Unclustered / Clustered / NonMonocyte</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>ResNet34</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>ImageNet</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G27" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>3-class single model</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>70</v>
+      </c>
+      <c r="J27" t="n">
+        <v>10</v>
+      </c>
+      <c r="K27" t="n">
+        <v>20</v>
+      </c>
+      <c r="L27" t="n">
+        <v>1200</v>
+      </c>
+      <c r="M27" t="n">
+        <v>3600</v>
+      </c>
+      <c r="N27" t="n">
+        <v>900</v>
+      </c>
+      <c r="O27" t="n">
+        <v>900</v>
+      </c>
+      <c r="P27" t="n">
+        <v>1800</v>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>Equal balance per class</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>AdamW</t>
+        </is>
+      </c>
+      <c r="S27" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="T27" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="U27" t="n">
+        <v>32</v>
+      </c>
+      <c r="V27" t="n">
+        <v>20</v>
+      </c>
+      <c r="W27" t="inlineStr">
+        <is>
+          <t>CosineAnnealingLR (T_max=20)</t>
+        </is>
+      </c>
+      <c r="X27" t="inlineStr">
+        <is>
+          <t>256x256</t>
+        </is>
+      </c>
+      <c r="Y27" t="inlineStr">
+        <is>
+          <t>HFlip, VFlip, Rotation(15°), ColorJitter(b=0.2,c=0.2), ImageNet norm</t>
+        </is>
+      </c>
+      <c r="Z27" t="n">
+        <v>0.8384</v>
+      </c>
+      <c r="AA27" t="n">
+        <v>0.722</v>
+      </c>
+      <c r="AB27" t="n">
+        <v>0.728</v>
+      </c>
+      <c r="AC27" t="n">
+        <v>0.725</v>
+      </c>
+      <c r="AD27" t="n">
+        <v>0.8453000000000001</v>
+      </c>
+      <c r="AE27" t="n">
+        <v>0.8642</v>
+      </c>
+      <c r="AF27" t="n">
+        <v>0.8547</v>
+      </c>
+      <c r="AG27" t="n">
+        <v>0.8836000000000001</v>
+      </c>
+      <c r="AH27" t="n">
+        <v>0.8628</v>
+      </c>
+      <c r="AI27" t="n">
+        <v>0.8731</v>
+      </c>
+      <c r="AJ27" t="n">
+        <v>0.8176</v>
+      </c>
+      <c r="AK27" t="n">
+        <v>0.8385</v>
+      </c>
+      <c r="AL27" t="n">
+        <v>0.8542</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
RBC count classifier + cleanup scripts
</commit_message>
<xml_diff>
--- a/experiment_log.xlsx
+++ b/experiment_log.xlsx
@@ -599,7 +599,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AO175"/>
+  <dimension ref="A1:AR199"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -24888,6 +24888,3639 @@
         <v>0.8391999999999999</v>
       </c>
     </row>
+    <row r="176">
+      <c r="A176" t="n">
+        <v>174</v>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>default config run</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>resnet34</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>ImageNet</t>
+        </is>
+      </c>
+      <c r="F176" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G176" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H176" t="inlineStr">
+        <is>
+          <t>RBC Count</t>
+        </is>
+      </c>
+      <c r="I176" t="n">
+        <v>70</v>
+      </c>
+      <c r="J176" t="n">
+        <v>10</v>
+      </c>
+      <c r="K176" t="n">
+        <v>20</v>
+      </c>
+      <c r="L176" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M176" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N176" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O176" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P176" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q176" t="inlineStr">
+        <is>
+          <t>Natural distribution</t>
+        </is>
+      </c>
+      <c r="R176" t="inlineStr">
+        <is>
+          <t>AdamW</t>
+        </is>
+      </c>
+      <c r="S176" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="T176" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="U176" t="n">
+        <v>32</v>
+      </c>
+      <c r="V176" t="n">
+        <v>20</v>
+      </c>
+      <c r="W176" t="inlineStr">
+        <is>
+          <t>CosineAnnealingLR (T_max=20)</t>
+        </is>
+      </c>
+      <c r="X176" t="inlineStr">
+        <is>
+          <t>256x256</t>
+        </is>
+      </c>
+      <c r="Y176" t="inlineStr">
+        <is>
+          <t>HFlip, VFlip, Rotation(15°), ColorJitter(b=0.2,c=0.2), ImageNet norm</t>
+        </is>
+      </c>
+      <c r="Z176" t="n">
+        <v>0.911</v>
+      </c>
+      <c r="AA176" t="n">
+        <v>0.9646</v>
+      </c>
+      <c r="AB176" t="n">
+        <v>0.9909</v>
+      </c>
+      <c r="AC176" t="n">
+        <v>0.9776</v>
+      </c>
+      <c r="AD176" t="n">
+        <v>0.8636</v>
+      </c>
+      <c r="AE176" t="n">
+        <v>0.7917</v>
+      </c>
+      <c r="AF176" t="n">
+        <v>0.8260999999999999</v>
+      </c>
+      <c r="AG176" t="n">
+        <v>0.8699</v>
+      </c>
+      <c r="AH176" t="n">
+        <v>0.9099</v>
+      </c>
+      <c r="AI176" t="n">
+        <v>0.9271</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="n">
+        <v>175</v>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>default config run</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>resnet34</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>ImageNet</t>
+        </is>
+      </c>
+      <c r="F177" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G177" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H177" t="inlineStr">
+        <is>
+          <t>RBC Count</t>
+        </is>
+      </c>
+      <c r="I177" t="n">
+        <v>70</v>
+      </c>
+      <c r="J177" t="n">
+        <v>10</v>
+      </c>
+      <c r="K177" t="n">
+        <v>20</v>
+      </c>
+      <c r="L177" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M177" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N177" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O177" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P177" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q177" t="inlineStr">
+        <is>
+          <t>Natural distribution</t>
+        </is>
+      </c>
+      <c r="R177" t="inlineStr">
+        <is>
+          <t>AdamW</t>
+        </is>
+      </c>
+      <c r="S177" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="T177" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="U177" t="n">
+        <v>32</v>
+      </c>
+      <c r="V177" t="n">
+        <v>20</v>
+      </c>
+      <c r="W177" t="inlineStr">
+        <is>
+          <t>CosineAnnealingLR (T_max=20)</t>
+        </is>
+      </c>
+      <c r="X177" t="inlineStr">
+        <is>
+          <t>256x256</t>
+        </is>
+      </c>
+      <c r="Y177" t="inlineStr">
+        <is>
+          <t>HFlip, VFlip, Rotation(15°), ColorJitter(b=0.2,c=0.2), ImageNet norm</t>
+        </is>
+      </c>
+      <c r="Z177" t="n">
+        <v>0.9267</v>
+      </c>
+      <c r="AA177" t="n">
+        <v>0.9560999999999999</v>
+      </c>
+      <c r="AB177" t="n">
+        <v>0.9909</v>
+      </c>
+      <c r="AC177" t="n">
+        <v>0.9732</v>
+      </c>
+      <c r="AD177" t="n">
+        <v>0.8696</v>
+      </c>
+      <c r="AE177" t="n">
+        <v>0.8333</v>
+      </c>
+      <c r="AF177" t="n">
+        <v>0.8511</v>
+      </c>
+      <c r="AG177" t="n">
+        <v>0.8998</v>
+      </c>
+      <c r="AH177" t="n">
+        <v>0.9255</v>
+      </c>
+      <c r="AI177" t="n">
+        <v>0.9062</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="n">
+        <v>176</v>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>resnet18</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>resnet18</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>ImageNet</t>
+        </is>
+      </c>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G178" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H178" t="inlineStr">
+        <is>
+          <t>RBC Count</t>
+        </is>
+      </c>
+      <c r="I178" t="n">
+        <v>70</v>
+      </c>
+      <c r="J178" t="n">
+        <v>10</v>
+      </c>
+      <c r="K178" t="n">
+        <v>20</v>
+      </c>
+      <c r="L178" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M178" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N178" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O178" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P178" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q178" t="inlineStr">
+        <is>
+          <t>Natural distribution</t>
+        </is>
+      </c>
+      <c r="R178" t="inlineStr">
+        <is>
+          <t>AdamW</t>
+        </is>
+      </c>
+      <c r="S178" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="T178" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="U178" t="n">
+        <v>32</v>
+      </c>
+      <c r="V178" t="n">
+        <v>20</v>
+      </c>
+      <c r="W178" t="inlineStr">
+        <is>
+          <t>CosineAnnealingLR (T_max=20)</t>
+        </is>
+      </c>
+      <c r="X178" t="inlineStr">
+        <is>
+          <t>256x256</t>
+        </is>
+      </c>
+      <c r="Y178" t="inlineStr">
+        <is>
+          <t>HFlip, VFlip, Rotation(15°), ColorJitter(b=0.2,c=0.2), ImageNet norm</t>
+        </is>
+      </c>
+      <c r="Z178" t="n">
+        <v>0.9162</v>
+      </c>
+      <c r="AA178" t="n">
+        <v>0.964</v>
+      </c>
+      <c r="AB178" t="n">
+        <v>0.9727</v>
+      </c>
+      <c r="AC178" t="n">
+        <v>0.9683</v>
+      </c>
+      <c r="AD178" t="n">
+        <v>0.881</v>
+      </c>
+      <c r="AE178" t="n">
+        <v>0.7708</v>
+      </c>
+      <c r="AF178" t="n">
+        <v>0.8222</v>
+      </c>
+      <c r="AG178" t="n">
+        <v>0.8879</v>
+      </c>
+      <c r="AH178" t="n">
+        <v>0.9152</v>
+      </c>
+      <c r="AI178" t="n">
+        <v>0.8542</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="n">
+        <v>177</v>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>resnet34</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>resnet34</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>ImageNet</t>
+        </is>
+      </c>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G179" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H179" t="inlineStr">
+        <is>
+          <t>RBC Count</t>
+        </is>
+      </c>
+      <c r="I179" t="n">
+        <v>70</v>
+      </c>
+      <c r="J179" t="n">
+        <v>10</v>
+      </c>
+      <c r="K179" t="n">
+        <v>20</v>
+      </c>
+      <c r="L179" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M179" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N179" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O179" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P179" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q179" t="inlineStr">
+        <is>
+          <t>Natural distribution</t>
+        </is>
+      </c>
+      <c r="R179" t="inlineStr">
+        <is>
+          <t>AdamW</t>
+        </is>
+      </c>
+      <c r="S179" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="T179" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="U179" t="n">
+        <v>32</v>
+      </c>
+      <c r="V179" t="n">
+        <v>20</v>
+      </c>
+      <c r="W179" t="inlineStr">
+        <is>
+          <t>CosineAnnealingLR (T_max=20)</t>
+        </is>
+      </c>
+      <c r="X179" t="inlineStr">
+        <is>
+          <t>256x256</t>
+        </is>
+      </c>
+      <c r="Y179" t="inlineStr">
+        <is>
+          <t>HFlip, VFlip, Rotation(15°), ColorJitter(b=0.2,c=0.2), ImageNet norm</t>
+        </is>
+      </c>
+      <c r="Z179" t="n">
+        <v>0.9267</v>
+      </c>
+      <c r="AA179" t="n">
+        <v>0.9727</v>
+      </c>
+      <c r="AB179" t="n">
+        <v>0.9727</v>
+      </c>
+      <c r="AC179" t="n">
+        <v>0.9727</v>
+      </c>
+      <c r="AD179" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="AE179" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="AF179" t="n">
+        <v>0.8571</v>
+      </c>
+      <c r="AG179" t="n">
+        <v>0.9016</v>
+      </c>
+      <c r="AH179" t="n">
+        <v>0.9268</v>
+      </c>
+      <c r="AI179" t="n">
+        <v>0.9062</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="n">
+        <v>178</v>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>resnet50</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>resnet50</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>ImageNet</t>
+        </is>
+      </c>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G180" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H180" t="inlineStr">
+        <is>
+          <t>RBC Count</t>
+        </is>
+      </c>
+      <c r="I180" t="n">
+        <v>70</v>
+      </c>
+      <c r="J180" t="n">
+        <v>10</v>
+      </c>
+      <c r="K180" t="n">
+        <v>20</v>
+      </c>
+      <c r="L180" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M180" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N180" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O180" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P180" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q180" t="inlineStr">
+        <is>
+          <t>Natural distribution</t>
+        </is>
+      </c>
+      <c r="R180" t="inlineStr">
+        <is>
+          <t>AdamW</t>
+        </is>
+      </c>
+      <c r="S180" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="T180" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="U180" t="n">
+        <v>32</v>
+      </c>
+      <c r="V180" t="n">
+        <v>20</v>
+      </c>
+      <c r="W180" t="inlineStr">
+        <is>
+          <t>CosineAnnealingLR (T_max=20)</t>
+        </is>
+      </c>
+      <c r="X180" t="inlineStr">
+        <is>
+          <t>256x256</t>
+        </is>
+      </c>
+      <c r="Y180" t="inlineStr">
+        <is>
+          <t>HFlip, VFlip, Rotation(15°), ColorJitter(b=0.2,c=0.2), ImageNet norm</t>
+        </is>
+      </c>
+      <c r="Z180" t="n">
+        <v>0.9372</v>
+      </c>
+      <c r="AA180" t="n">
+        <v>0.9815</v>
+      </c>
+      <c r="AB180" t="n">
+        <v>0.9636</v>
+      </c>
+      <c r="AC180" t="n">
+        <v>0.9725</v>
+      </c>
+      <c r="AD180" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="AE180" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="AF180" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="AG180" t="n">
+        <v>0.9197</v>
+      </c>
+      <c r="AH180" t="n">
+        <v>0.9375</v>
+      </c>
+      <c r="AI180" t="n">
+        <v>0.9062</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="n">
+        <v>179</v>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>resnet101</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>resnet101</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>ImageNet</t>
+        </is>
+      </c>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G181" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H181" t="inlineStr">
+        <is>
+          <t>RBC Count</t>
+        </is>
+      </c>
+      <c r="I181" t="n">
+        <v>70</v>
+      </c>
+      <c r="J181" t="n">
+        <v>10</v>
+      </c>
+      <c r="K181" t="n">
+        <v>20</v>
+      </c>
+      <c r="L181" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M181" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N181" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O181" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P181" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q181" t="inlineStr">
+        <is>
+          <t>Natural distribution</t>
+        </is>
+      </c>
+      <c r="R181" t="inlineStr">
+        <is>
+          <t>AdamW</t>
+        </is>
+      </c>
+      <c r="S181" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="T181" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="U181" t="n">
+        <v>32</v>
+      </c>
+      <c r="V181" t="n">
+        <v>20</v>
+      </c>
+      <c r="W181" t="inlineStr">
+        <is>
+          <t>CosineAnnealingLR (T_max=20)</t>
+        </is>
+      </c>
+      <c r="X181" t="inlineStr">
+        <is>
+          <t>256x256</t>
+        </is>
+      </c>
+      <c r="Y181" t="inlineStr">
+        <is>
+          <t>HFlip, VFlip, Rotation(15°), ColorJitter(b=0.2,c=0.2), ImageNet norm</t>
+        </is>
+      </c>
+      <c r="Z181" t="n">
+        <v>0.9005</v>
+      </c>
+      <c r="AA181" t="n">
+        <v>0.9808</v>
+      </c>
+      <c r="AB181" t="n">
+        <v>0.9273</v>
+      </c>
+      <c r="AC181" t="n">
+        <v>0.9533</v>
+      </c>
+      <c r="AD181" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="AE181" t="n">
+        <v>0.8333</v>
+      </c>
+      <c r="AF181" t="n">
+        <v>0.8163</v>
+      </c>
+      <c r="AG181" t="n">
+        <v>0.8756</v>
+      </c>
+      <c r="AH181" t="n">
+        <v>0.9022</v>
+      </c>
+      <c r="AI181" t="n">
+        <v>0.9271</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="n">
+        <v>180</v>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>resnet152</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>resnet152</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>ImageNet</t>
+        </is>
+      </c>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G182" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H182" t="inlineStr">
+        <is>
+          <t>RBC Count</t>
+        </is>
+      </c>
+      <c r="I182" t="n">
+        <v>70</v>
+      </c>
+      <c r="J182" t="n">
+        <v>10</v>
+      </c>
+      <c r="K182" t="n">
+        <v>20</v>
+      </c>
+      <c r="L182" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M182" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N182" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O182" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P182" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q182" t="inlineStr">
+        <is>
+          <t>Natural distribution</t>
+        </is>
+      </c>
+      <c r="R182" t="inlineStr">
+        <is>
+          <t>AdamW</t>
+        </is>
+      </c>
+      <c r="S182" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="T182" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="U182" t="n">
+        <v>32</v>
+      </c>
+      <c r="V182" t="n">
+        <v>20</v>
+      </c>
+      <c r="W182" t="inlineStr">
+        <is>
+          <t>CosineAnnealingLR (T_max=20)</t>
+        </is>
+      </c>
+      <c r="X182" t="inlineStr">
+        <is>
+          <t>256x256</t>
+        </is>
+      </c>
+      <c r="Y182" t="inlineStr">
+        <is>
+          <t>HFlip, VFlip, Rotation(15°), ColorJitter(b=0.2,c=0.2), ImageNet norm</t>
+        </is>
+      </c>
+      <c r="Z182" t="n">
+        <v>0.9215</v>
+      </c>
+      <c r="AA182" t="n">
+        <v>0.9558</v>
+      </c>
+      <c r="AB182" t="n">
+        <v>0.9818</v>
+      </c>
+      <c r="AC182" t="n">
+        <v>0.9686</v>
+      </c>
+      <c r="AD182" t="n">
+        <v>0.8696</v>
+      </c>
+      <c r="AE182" t="n">
+        <v>0.8333</v>
+      </c>
+      <c r="AF182" t="n">
+        <v>0.8511</v>
+      </c>
+      <c r="AG182" t="n">
+        <v>0.8937</v>
+      </c>
+      <c r="AH182" t="n">
+        <v>0.9206</v>
+      </c>
+      <c r="AI182" t="n">
+        <v>0.9271</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="n">
+        <v>181</v>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>efficientnet_b0</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>efficientnet_b0</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>ImageNet</t>
+        </is>
+      </c>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G183" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H183" t="inlineStr">
+        <is>
+          <t>RBC Count</t>
+        </is>
+      </c>
+      <c r="I183" t="n">
+        <v>70</v>
+      </c>
+      <c r="J183" t="n">
+        <v>10</v>
+      </c>
+      <c r="K183" t="n">
+        <v>20</v>
+      </c>
+      <c r="L183" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M183" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N183" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O183" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P183" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q183" t="inlineStr">
+        <is>
+          <t>Natural distribution</t>
+        </is>
+      </c>
+      <c r="R183" t="inlineStr">
+        <is>
+          <t>AdamW</t>
+        </is>
+      </c>
+      <c r="S183" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="T183" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="U183" t="n">
+        <v>32</v>
+      </c>
+      <c r="V183" t="n">
+        <v>20</v>
+      </c>
+      <c r="W183" t="inlineStr">
+        <is>
+          <t>CosineAnnealingLR (T_max=20)</t>
+        </is>
+      </c>
+      <c r="X183" t="inlineStr">
+        <is>
+          <t>256x256</t>
+        </is>
+      </c>
+      <c r="Y183" t="inlineStr">
+        <is>
+          <t>HFlip, VFlip, Rotation(15°), ColorJitter(b=0.2,c=0.2), ImageNet norm</t>
+        </is>
+      </c>
+      <c r="Z183" t="n">
+        <v>0.8743</v>
+      </c>
+      <c r="AA183" t="n">
+        <v>0.9137999999999999</v>
+      </c>
+      <c r="AB183" t="n">
+        <v>0.9636</v>
+      </c>
+      <c r="AC183" t="n">
+        <v>0.9381</v>
+      </c>
+      <c r="AD183" t="n">
+        <v>0.825</v>
+      </c>
+      <c r="AE183" t="n">
+        <v>0.6875</v>
+      </c>
+      <c r="AF183" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="AG183" t="n">
+        <v>0.8372000000000001</v>
+      </c>
+      <c r="AH183" t="n">
+        <v>0.871</v>
+      </c>
+      <c r="AI183" t="n">
+        <v>0.8958</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="n">
+        <v>182</v>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>efficientnet_b1</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>efficientnet_b1</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>ImageNet</t>
+        </is>
+      </c>
+      <c r="F184" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G184" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H184" t="inlineStr">
+        <is>
+          <t>RBC Count</t>
+        </is>
+      </c>
+      <c r="I184" t="n">
+        <v>70</v>
+      </c>
+      <c r="J184" t="n">
+        <v>10</v>
+      </c>
+      <c r="K184" t="n">
+        <v>20</v>
+      </c>
+      <c r="L184" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M184" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N184" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O184" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P184" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q184" t="inlineStr">
+        <is>
+          <t>Natural distribution</t>
+        </is>
+      </c>
+      <c r="R184" t="inlineStr">
+        <is>
+          <t>AdamW</t>
+        </is>
+      </c>
+      <c r="S184" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="T184" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="U184" t="n">
+        <v>32</v>
+      </c>
+      <c r="V184" t="n">
+        <v>20</v>
+      </c>
+      <c r="W184" t="inlineStr">
+        <is>
+          <t>CosineAnnealingLR (T_max=20)</t>
+        </is>
+      </c>
+      <c r="X184" t="inlineStr">
+        <is>
+          <t>256x256</t>
+        </is>
+      </c>
+      <c r="Y184" t="inlineStr">
+        <is>
+          <t>HFlip, VFlip, Rotation(15°), ColorJitter(b=0.2,c=0.2), ImageNet norm</t>
+        </is>
+      </c>
+      <c r="Z184" t="n">
+        <v>0.822</v>
+      </c>
+      <c r="AA184" t="n">
+        <v>0.8793</v>
+      </c>
+      <c r="AB184" t="n">
+        <v>0.9273</v>
+      </c>
+      <c r="AC184" t="n">
+        <v>0.9026999999999999</v>
+      </c>
+      <c r="AD184" t="n">
+        <v>0.7576000000000001</v>
+      </c>
+      <c r="AE184" t="n">
+        <v>0.5208</v>
+      </c>
+      <c r="AF184" t="n">
+        <v>0.6173</v>
+      </c>
+      <c r="AG184" t="n">
+        <v>0.7733</v>
+      </c>
+      <c r="AH184" t="n">
+        <v>0.8132</v>
+      </c>
+      <c r="AI184" t="n">
+        <v>0.8125</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="n">
+        <v>183</v>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>efficientnet_b4</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>efficientnet_b4</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>ImageNet</t>
+        </is>
+      </c>
+      <c r="F185" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G185" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H185" t="inlineStr">
+        <is>
+          <t>RBC Count</t>
+        </is>
+      </c>
+      <c r="I185" t="n">
+        <v>70</v>
+      </c>
+      <c r="J185" t="n">
+        <v>10</v>
+      </c>
+      <c r="K185" t="n">
+        <v>20</v>
+      </c>
+      <c r="L185" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M185" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N185" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O185" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P185" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q185" t="inlineStr">
+        <is>
+          <t>Natural distribution</t>
+        </is>
+      </c>
+      <c r="R185" t="inlineStr">
+        <is>
+          <t>AdamW</t>
+        </is>
+      </c>
+      <c r="S185" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="T185" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="U185" t="n">
+        <v>32</v>
+      </c>
+      <c r="V185" t="n">
+        <v>20</v>
+      </c>
+      <c r="W185" t="inlineStr">
+        <is>
+          <t>CosineAnnealingLR (T_max=20)</t>
+        </is>
+      </c>
+      <c r="X185" t="inlineStr">
+        <is>
+          <t>256x256</t>
+        </is>
+      </c>
+      <c r="Y185" t="inlineStr">
+        <is>
+          <t>HFlip, VFlip, Rotation(15°), ColorJitter(b=0.2,c=0.2), ImageNet norm</t>
+        </is>
+      </c>
+      <c r="Z185" t="n">
+        <v>0.8429</v>
+      </c>
+      <c r="AA185" t="n">
+        <v>0.8699</v>
+      </c>
+      <c r="AB185" t="n">
+        <v>0.9727</v>
+      </c>
+      <c r="AC185" t="n">
+        <v>0.9185</v>
+      </c>
+      <c r="AD185" t="n">
+        <v>0.8276</v>
+      </c>
+      <c r="AE185" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AF185" t="n">
+        <v>0.6234</v>
+      </c>
+      <c r="AG185" t="n">
+        <v>0.7917</v>
+      </c>
+      <c r="AH185" t="n">
+        <v>0.8296</v>
+      </c>
+      <c r="AI185" t="n">
+        <v>0.8229</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="n">
+        <v>184</v>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>convnext_tiny</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>convnext_tiny</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>ImageNet</t>
+        </is>
+      </c>
+      <c r="F186" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G186" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H186" t="inlineStr">
+        <is>
+          <t>RBC Count</t>
+        </is>
+      </c>
+      <c r="I186" t="n">
+        <v>70</v>
+      </c>
+      <c r="J186" t="n">
+        <v>10</v>
+      </c>
+      <c r="K186" t="n">
+        <v>20</v>
+      </c>
+      <c r="L186" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M186" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N186" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O186" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P186" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q186" t="inlineStr">
+        <is>
+          <t>Natural distribution</t>
+        </is>
+      </c>
+      <c r="R186" t="inlineStr">
+        <is>
+          <t>AdamW</t>
+        </is>
+      </c>
+      <c r="S186" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="T186" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="U186" t="n">
+        <v>32</v>
+      </c>
+      <c r="V186" t="n">
+        <v>20</v>
+      </c>
+      <c r="W186" t="inlineStr">
+        <is>
+          <t>CosineAnnealingLR (T_max=20)</t>
+        </is>
+      </c>
+      <c r="X186" t="inlineStr">
+        <is>
+          <t>256x256</t>
+        </is>
+      </c>
+      <c r="Y186" t="inlineStr">
+        <is>
+          <t>HFlip, VFlip, Rotation(15°), ColorJitter(b=0.2,c=0.2), ImageNet norm</t>
+        </is>
+      </c>
+      <c r="Z186" t="n">
+        <v>0.9215</v>
+      </c>
+      <c r="AA186" t="n">
+        <v>0.9560999999999999</v>
+      </c>
+      <c r="AB186" t="n">
+        <v>0.9909</v>
+      </c>
+      <c r="AC186" t="n">
+        <v>0.9732</v>
+      </c>
+      <c r="AD186" t="n">
+        <v>0.9231</v>
+      </c>
+      <c r="AE186" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="AF186" t="n">
+        <v>0.8276</v>
+      </c>
+      <c r="AG186" t="n">
+        <v>0.8913</v>
+      </c>
+      <c r="AH186" t="n">
+        <v>0.9193</v>
+      </c>
+      <c r="AI186" t="n">
+        <v>0.9375</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="n">
+        <v>185</v>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>convnext_base</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>convnext_base</t>
+        </is>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>ImageNet</t>
+        </is>
+      </c>
+      <c r="F187" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G187" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H187" t="inlineStr">
+        <is>
+          <t>RBC Count</t>
+        </is>
+      </c>
+      <c r="I187" t="n">
+        <v>70</v>
+      </c>
+      <c r="J187" t="n">
+        <v>10</v>
+      </c>
+      <c r="K187" t="n">
+        <v>20</v>
+      </c>
+      <c r="L187" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M187" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N187" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O187" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P187" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q187" t="inlineStr">
+        <is>
+          <t>Natural distribution</t>
+        </is>
+      </c>
+      <c r="R187" t="inlineStr">
+        <is>
+          <t>AdamW</t>
+        </is>
+      </c>
+      <c r="S187" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="T187" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="U187" t="n">
+        <v>32</v>
+      </c>
+      <c r="V187" t="n">
+        <v>20</v>
+      </c>
+      <c r="W187" t="inlineStr">
+        <is>
+          <t>CosineAnnealingLR (T_max=20)</t>
+        </is>
+      </c>
+      <c r="X187" t="inlineStr">
+        <is>
+          <t>256x256</t>
+        </is>
+      </c>
+      <c r="Y187" t="inlineStr">
+        <is>
+          <t>HFlip, VFlip, Rotation(15°), ColorJitter(b=0.2,c=0.2), ImageNet norm</t>
+        </is>
+      </c>
+      <c r="Z187" t="n">
+        <v>0.9319</v>
+      </c>
+      <c r="AA187" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB187" t="n">
+        <v>0.9818</v>
+      </c>
+      <c r="AC187" t="n">
+        <v>0.9908</v>
+      </c>
+      <c r="AD187" t="n">
+        <v>0.8431</v>
+      </c>
+      <c r="AE187" t="n">
+        <v>0.8958</v>
+      </c>
+      <c r="AF187" t="n">
+        <v>0.8687</v>
+      </c>
+      <c r="AG187" t="n">
+        <v>0.8968</v>
+      </c>
+      <c r="AH187" t="n">
+        <v>0.9325</v>
+      </c>
+      <c r="AI187" t="n">
+        <v>0.9271</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="n">
+        <v>186</v>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>vit_b16</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>vit_b16</t>
+        </is>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>ImageNet</t>
+        </is>
+      </c>
+      <c r="F188" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G188" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H188" t="inlineStr">
+        <is>
+          <t>RBC Count</t>
+        </is>
+      </c>
+      <c r="I188" t="n">
+        <v>70</v>
+      </c>
+      <c r="J188" t="n">
+        <v>10</v>
+      </c>
+      <c r="K188" t="n">
+        <v>20</v>
+      </c>
+      <c r="L188" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M188" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N188" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O188" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P188" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q188" t="inlineStr">
+        <is>
+          <t>Natural distribution</t>
+        </is>
+      </c>
+      <c r="R188" t="inlineStr">
+        <is>
+          <t>AdamW</t>
+        </is>
+      </c>
+      <c r="S188" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="T188" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="U188" t="n">
+        <v>32</v>
+      </c>
+      <c r="V188" t="n">
+        <v>20</v>
+      </c>
+      <c r="W188" t="inlineStr">
+        <is>
+          <t>CosineAnnealingLR (T_max=20)</t>
+        </is>
+      </c>
+      <c r="X188" t="inlineStr">
+        <is>
+          <t>256x256</t>
+        </is>
+      </c>
+      <c r="Y188" t="inlineStr">
+        <is>
+          <t>HFlip, VFlip, Rotation(15°), ColorJitter(b=0.2,c=0.2), ImageNet norm</t>
+        </is>
+      </c>
+      <c r="Z188" t="n">
+        <v>0.9005</v>
+      </c>
+      <c r="AA188" t="n">
+        <v>0.9397</v>
+      </c>
+      <c r="AB188" t="n">
+        <v>0.9909</v>
+      </c>
+      <c r="AC188" t="n">
+        <v>0.9646</v>
+      </c>
+      <c r="AD188" t="n">
+        <v>0.8372000000000001</v>
+      </c>
+      <c r="AE188" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="AF188" t="n">
+        <v>0.7912</v>
+      </c>
+      <c r="AG188" t="n">
+        <v>0.8622</v>
+      </c>
+      <c r="AH188" t="n">
+        <v>0.8979</v>
+      </c>
+      <c r="AI188" t="n">
+        <v>0.9062</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="n">
+        <v>187</v>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>resnet18</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>resnet18</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>ImageNet</t>
+        </is>
+      </c>
+      <c r="F189" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G189" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H189" t="inlineStr">
+        <is>
+          <t>Clustered RBC Count</t>
+        </is>
+      </c>
+      <c r="I189" t="n">
+        <v>70</v>
+      </c>
+      <c r="J189" t="n">
+        <v>10</v>
+      </c>
+      <c r="K189" t="n">
+        <v>20</v>
+      </c>
+      <c r="L189" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M189" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N189" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O189" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P189" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q189" t="inlineStr">
+        <is>
+          <t>WeightedRandomSampler equal balance</t>
+        </is>
+      </c>
+      <c r="R189" t="inlineStr">
+        <is>
+          <t>AdamW</t>
+        </is>
+      </c>
+      <c r="S189" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="T189" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="U189" t="n">
+        <v>32</v>
+      </c>
+      <c r="V189" t="n">
+        <v>20</v>
+      </c>
+      <c r="W189" t="inlineStr">
+        <is>
+          <t>CosineAnnealingLR (T_max=20)</t>
+        </is>
+      </c>
+      <c r="X189" t="inlineStr">
+        <is>
+          <t>256x256</t>
+        </is>
+      </c>
+      <c r="Y189" t="inlineStr">
+        <is>
+          <t>HFlip, VFlip, Rotation(15°), ColorJitter(b=0.2,c=0.2), ImageNet norm</t>
+        </is>
+      </c>
+      <c r="Z189" t="n">
+        <v>0.9216</v>
+      </c>
+      <c r="AA189" t="n">
+        <v>0.9927</v>
+      </c>
+      <c r="AB189" t="n">
+        <v>0.9617</v>
+      </c>
+      <c r="AC189" t="n">
+        <v>0.977</v>
+      </c>
+      <c r="AD189" t="n">
+        <v>0.8506</v>
+      </c>
+      <c r="AE189" t="n">
+        <v>0.7957</v>
+      </c>
+      <c r="AF189" t="n">
+        <v>0.8222</v>
+      </c>
+      <c r="AG189" t="n">
+        <v>0.6842</v>
+      </c>
+      <c r="AH189" t="n">
+        <v>0.7065</v>
+      </c>
+      <c r="AI189" t="n">
+        <v>0.6952</v>
+      </c>
+      <c r="AJ189" t="n">
+        <v>0.8095</v>
+      </c>
+      <c r="AK189" t="n">
+        <v>0.8643999999999999</v>
+      </c>
+      <c r="AL189" t="n">
+        <v>0.8361</v>
+      </c>
+      <c r="AM189" t="n">
+        <v>0.7432</v>
+      </c>
+      <c r="AN189" t="n">
+        <v>0.9821</v>
+      </c>
+      <c r="AO189" t="n">
+        <v>0.8462</v>
+      </c>
+      <c r="AP189" t="n">
+        <v>0.8353</v>
+      </c>
+      <c r="AQ189" t="n">
+        <v>0.9231</v>
+      </c>
+      <c r="AR189" t="n">
+        <v>0.9208</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="n">
+        <v>188</v>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>resnet34</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>resnet34</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>ImageNet</t>
+        </is>
+      </c>
+      <c r="F190" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G190" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H190" t="inlineStr">
+        <is>
+          <t>Clustered RBC Count</t>
+        </is>
+      </c>
+      <c r="I190" t="n">
+        <v>70</v>
+      </c>
+      <c r="J190" t="n">
+        <v>10</v>
+      </c>
+      <c r="K190" t="n">
+        <v>20</v>
+      </c>
+      <c r="L190" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M190" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N190" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O190" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P190" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q190" t="inlineStr">
+        <is>
+          <t>WeightedRandomSampler equal balance</t>
+        </is>
+      </c>
+      <c r="R190" t="inlineStr">
+        <is>
+          <t>AdamW</t>
+        </is>
+      </c>
+      <c r="S190" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="T190" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="U190" t="n">
+        <v>32</v>
+      </c>
+      <c r="V190" t="n">
+        <v>20</v>
+      </c>
+      <c r="W190" t="inlineStr">
+        <is>
+          <t>CosineAnnealingLR (T_max=20)</t>
+        </is>
+      </c>
+      <c r="X190" t="inlineStr">
+        <is>
+          <t>256x256</t>
+        </is>
+      </c>
+      <c r="Y190" t="inlineStr">
+        <is>
+          <t>HFlip, VFlip, Rotation(15°), ColorJitter(b=0.2,c=0.2), ImageNet norm</t>
+        </is>
+      </c>
+      <c r="Z190" t="n">
+        <v>0.9362</v>
+      </c>
+      <c r="AA190" t="n">
+        <v>0.9887</v>
+      </c>
+      <c r="AB190" t="n">
+        <v>0.9708</v>
+      </c>
+      <c r="AC190" t="n">
+        <v>0.9797</v>
+      </c>
+      <c r="AD190" t="n">
+        <v>0.9012</v>
+      </c>
+      <c r="AE190" t="n">
+        <v>0.8333</v>
+      </c>
+      <c r="AF190" t="n">
+        <v>0.8659</v>
+      </c>
+      <c r="AG190" t="n">
+        <v>0.7727000000000001</v>
+      </c>
+      <c r="AH190" t="n">
+        <v>0.7391</v>
+      </c>
+      <c r="AI190" t="n">
+        <v>0.7556</v>
+      </c>
+      <c r="AJ190" t="n">
+        <v>0.7639</v>
+      </c>
+      <c r="AK190" t="n">
+        <v>0.9322</v>
+      </c>
+      <c r="AL190" t="n">
+        <v>0.8397</v>
+      </c>
+      <c r="AM190" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="AN190" t="n">
+        <v>0.9643</v>
+      </c>
+      <c r="AO190" t="n">
+        <v>0.8745000000000001</v>
+      </c>
+      <c r="AP190" t="n">
+        <v>0.8631</v>
+      </c>
+      <c r="AQ190" t="n">
+        <v>0.9368</v>
+      </c>
+      <c r="AR190" t="n">
+        <v>0.9347</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="n">
+        <v>189</v>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>resnet50</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>resnet50</t>
+        </is>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>ImageNet</t>
+        </is>
+      </c>
+      <c r="F191" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G191" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H191" t="inlineStr">
+        <is>
+          <t>Clustered RBC Count</t>
+        </is>
+      </c>
+      <c r="I191" t="n">
+        <v>70</v>
+      </c>
+      <c r="J191" t="n">
+        <v>10</v>
+      </c>
+      <c r="K191" t="n">
+        <v>20</v>
+      </c>
+      <c r="L191" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M191" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N191" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O191" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P191" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q191" t="inlineStr">
+        <is>
+          <t>WeightedRandomSampler equal balance</t>
+        </is>
+      </c>
+      <c r="R191" t="inlineStr">
+        <is>
+          <t>AdamW</t>
+        </is>
+      </c>
+      <c r="S191" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="T191" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="U191" t="n">
+        <v>32</v>
+      </c>
+      <c r="V191" t="n">
+        <v>20</v>
+      </c>
+      <c r="W191" t="inlineStr">
+        <is>
+          <t>CosineAnnealingLR (T_max=20)</t>
+        </is>
+      </c>
+      <c r="X191" t="inlineStr">
+        <is>
+          <t>256x256</t>
+        </is>
+      </c>
+      <c r="Y191" t="inlineStr">
+        <is>
+          <t>HFlip, VFlip, Rotation(15°), ColorJitter(b=0.2,c=0.2), ImageNet norm</t>
+        </is>
+      </c>
+      <c r="Z191" t="n">
+        <v>0.9348</v>
+      </c>
+      <c r="AA191" t="n">
+        <v>0.9948</v>
+      </c>
+      <c r="AB191" t="n">
+        <v>0.9667</v>
+      </c>
+      <c r="AC191" t="n">
+        <v>0.9806</v>
+      </c>
+      <c r="AD191" t="n">
+        <v>0.8441</v>
+      </c>
+      <c r="AE191" t="n">
+        <v>0.8441</v>
+      </c>
+      <c r="AF191" t="n">
+        <v>0.8441</v>
+      </c>
+      <c r="AG191" t="n">
+        <v>0.7711</v>
+      </c>
+      <c r="AH191" t="n">
+        <v>0.6957</v>
+      </c>
+      <c r="AI191" t="n">
+        <v>0.7314000000000001</v>
+      </c>
+      <c r="AJ191" t="n">
+        <v>0.7808</v>
+      </c>
+      <c r="AK191" t="n">
+        <v>0.9661</v>
+      </c>
+      <c r="AL191" t="n">
+        <v>0.8636</v>
+      </c>
+      <c r="AM191" t="n">
+        <v>0.8148</v>
+      </c>
+      <c r="AN191" t="n">
+        <v>0.9821</v>
+      </c>
+      <c r="AO191" t="n">
+        <v>0.8907</v>
+      </c>
+      <c r="AP191" t="n">
+        <v>0.8621</v>
+      </c>
+      <c r="AQ191" t="n">
+        <v>0.9353</v>
+      </c>
+      <c r="AR191" t="n">
+        <v>0.9347</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="n">
+        <v>190</v>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>resnet101</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>resnet101</t>
+        </is>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>ImageNet</t>
+        </is>
+      </c>
+      <c r="F192" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G192" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H192" t="inlineStr">
+        <is>
+          <t>Clustered RBC Count</t>
+        </is>
+      </c>
+      <c r="I192" t="n">
+        <v>70</v>
+      </c>
+      <c r="J192" t="n">
+        <v>10</v>
+      </c>
+      <c r="K192" t="n">
+        <v>20</v>
+      </c>
+      <c r="L192" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M192" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N192" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O192" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P192" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q192" t="inlineStr">
+        <is>
+          <t>WeightedRandomSampler equal balance</t>
+        </is>
+      </c>
+      <c r="R192" t="inlineStr">
+        <is>
+          <t>AdamW</t>
+        </is>
+      </c>
+      <c r="S192" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="T192" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="U192" t="n">
+        <v>32</v>
+      </c>
+      <c r="V192" t="n">
+        <v>20</v>
+      </c>
+      <c r="W192" t="inlineStr">
+        <is>
+          <t>CosineAnnealingLR (T_max=20)</t>
+        </is>
+      </c>
+      <c r="X192" t="inlineStr">
+        <is>
+          <t>256x256</t>
+        </is>
+      </c>
+      <c r="Y192" t="inlineStr">
+        <is>
+          <t>HFlip, VFlip, Rotation(15°), ColorJitter(b=0.2,c=0.2), ImageNet norm</t>
+        </is>
+      </c>
+      <c r="Z192" t="n">
+        <v>0.9292</v>
+      </c>
+      <c r="AA192" t="n">
+        <v>0.9827</v>
+      </c>
+      <c r="AB192" t="n">
+        <v>0.9708</v>
+      </c>
+      <c r="AC192" t="n">
+        <v>0.9767</v>
+      </c>
+      <c r="AD192" t="n">
+        <v>0.8772</v>
+      </c>
+      <c r="AE192" t="n">
+        <v>0.8065</v>
+      </c>
+      <c r="AF192" t="n">
+        <v>0.8403</v>
+      </c>
+      <c r="AG192" t="n">
+        <v>0.6931</v>
+      </c>
+      <c r="AH192" t="n">
+        <v>0.7609</v>
+      </c>
+      <c r="AI192" t="n">
+        <v>0.7254</v>
+      </c>
+      <c r="AJ192" t="n">
+        <v>0.8333</v>
+      </c>
+      <c r="AK192" t="n">
+        <v>0.8475</v>
+      </c>
+      <c r="AL192" t="n">
+        <v>0.8403</v>
+      </c>
+      <c r="AM192" t="n">
+        <v>0.8217</v>
+      </c>
+      <c r="AN192" t="n">
+        <v>0.9464</v>
+      </c>
+      <c r="AO192" t="n">
+        <v>0.8797</v>
+      </c>
+      <c r="AP192" t="n">
+        <v>0.8525</v>
+      </c>
+      <c r="AQ192" t="n">
+        <v>0.9298999999999999</v>
+      </c>
+      <c r="AR192" t="n">
+        <v>0.9458</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="n">
+        <v>191</v>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>resnet152</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>resnet152</t>
+        </is>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>ImageNet</t>
+        </is>
+      </c>
+      <c r="F193" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G193" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H193" t="inlineStr">
+        <is>
+          <t>Clustered RBC Count</t>
+        </is>
+      </c>
+      <c r="I193" t="n">
+        <v>70</v>
+      </c>
+      <c r="J193" t="n">
+        <v>10</v>
+      </c>
+      <c r="K193" t="n">
+        <v>20</v>
+      </c>
+      <c r="L193" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M193" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N193" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O193" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P193" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q193" t="inlineStr">
+        <is>
+          <t>WeightedRandomSampler equal balance</t>
+        </is>
+      </c>
+      <c r="R193" t="inlineStr">
+        <is>
+          <t>AdamW</t>
+        </is>
+      </c>
+      <c r="S193" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="T193" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="U193" t="n">
+        <v>32</v>
+      </c>
+      <c r="V193" t="n">
+        <v>20</v>
+      </c>
+      <c r="W193" t="inlineStr">
+        <is>
+          <t>CosineAnnealingLR (T_max=20)</t>
+        </is>
+      </c>
+      <c r="X193" t="inlineStr">
+        <is>
+          <t>256x256</t>
+        </is>
+      </c>
+      <c r="Y193" t="inlineStr">
+        <is>
+          <t>HFlip, VFlip, Rotation(15°), ColorJitter(b=0.2,c=0.2), ImageNet norm</t>
+        </is>
+      </c>
+      <c r="Z193" t="n">
+        <v>0.9298999999999999</v>
+      </c>
+      <c r="AA193" t="n">
+        <v>0.9917</v>
+      </c>
+      <c r="AB193" t="n">
+        <v>0.9647</v>
+      </c>
+      <c r="AC193" t="n">
+        <v>0.978</v>
+      </c>
+      <c r="AD193" t="n">
+        <v>0.8736</v>
+      </c>
+      <c r="AE193" t="n">
+        <v>0.8172</v>
+      </c>
+      <c r="AF193" t="n">
+        <v>0.8444</v>
+      </c>
+      <c r="AG193" t="n">
+        <v>0.6887</v>
+      </c>
+      <c r="AH193" t="n">
+        <v>0.7935</v>
+      </c>
+      <c r="AI193" t="n">
+        <v>0.7374000000000001</v>
+      </c>
+      <c r="AJ193" t="n">
+        <v>0.8475</v>
+      </c>
+      <c r="AK193" t="n">
+        <v>0.8475</v>
+      </c>
+      <c r="AL193" t="n">
+        <v>0.8475</v>
+      </c>
+      <c r="AM193" t="n">
+        <v>0.7883</v>
+      </c>
+      <c r="AN193" t="n">
+        <v>0.9643</v>
+      </c>
+      <c r="AO193" t="n">
+        <v>0.8675</v>
+      </c>
+      <c r="AP193" t="n">
+        <v>0.855</v>
+      </c>
+      <c r="AQ193" t="n">
+        <v>0.9315</v>
+      </c>
+      <c r="AR193" t="n">
+        <v>0.9361</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="n">
+        <v>192</v>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>efficientnet_b0</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>efficientnet_b0</t>
+        </is>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>ImageNet</t>
+        </is>
+      </c>
+      <c r="F194" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G194" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H194" t="inlineStr">
+        <is>
+          <t>Clustered RBC Count</t>
+        </is>
+      </c>
+      <c r="I194" t="n">
+        <v>70</v>
+      </c>
+      <c r="J194" t="n">
+        <v>10</v>
+      </c>
+      <c r="K194" t="n">
+        <v>20</v>
+      </c>
+      <c r="L194" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M194" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N194" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O194" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P194" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q194" t="inlineStr">
+        <is>
+          <t>WeightedRandomSampler equal balance</t>
+        </is>
+      </c>
+      <c r="R194" t="inlineStr">
+        <is>
+          <t>AdamW</t>
+        </is>
+      </c>
+      <c r="S194" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="T194" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="U194" t="n">
+        <v>32</v>
+      </c>
+      <c r="V194" t="n">
+        <v>20</v>
+      </c>
+      <c r="W194" t="inlineStr">
+        <is>
+          <t>CosineAnnealingLR (T_max=20)</t>
+        </is>
+      </c>
+      <c r="X194" t="inlineStr">
+        <is>
+          <t>256x256</t>
+        </is>
+      </c>
+      <c r="Y194" t="inlineStr">
+        <is>
+          <t>HFlip, VFlip, Rotation(15°), ColorJitter(b=0.2,c=0.2), ImageNet norm</t>
+        </is>
+      </c>
+      <c r="Z194" t="n">
+        <v>0.8931</v>
+      </c>
+      <c r="AA194" t="n">
+        <v>0.9864000000000001</v>
+      </c>
+      <c r="AB194" t="n">
+        <v>0.9496</v>
+      </c>
+      <c r="AC194" t="n">
+        <v>0.9676</v>
+      </c>
+      <c r="AD194" t="n">
+        <v>0.7302</v>
+      </c>
+      <c r="AE194" t="n">
+        <v>0.7419</v>
+      </c>
+      <c r="AF194" t="n">
+        <v>0.736</v>
+      </c>
+      <c r="AG194" t="n">
+        <v>0.5259</v>
+      </c>
+      <c r="AH194" t="n">
+        <v>0.663</v>
+      </c>
+      <c r="AI194" t="n">
+        <v>0.5865</v>
+      </c>
+      <c r="AJ194" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="AK194" t="n">
+        <v>0.8305</v>
+      </c>
+      <c r="AL194" t="n">
+        <v>0.7597</v>
+      </c>
+      <c r="AM194" t="n">
+        <v>0.8739</v>
+      </c>
+      <c r="AN194" t="n">
+        <v>0.8661</v>
+      </c>
+      <c r="AO194" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="AP194" t="n">
+        <v>0.784</v>
+      </c>
+      <c r="AQ194" t="n">
+        <v>0.8973</v>
+      </c>
+      <c r="AR194" t="n">
+        <v>0.9139</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="n">
+        <v>193</v>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>efficientnet_b1</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>efficientnet_b1</t>
+        </is>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>ImageNet</t>
+        </is>
+      </c>
+      <c r="F195" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G195" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H195" t="inlineStr">
+        <is>
+          <t>Clustered RBC Count</t>
+        </is>
+      </c>
+      <c r="I195" t="n">
+        <v>70</v>
+      </c>
+      <c r="J195" t="n">
+        <v>10</v>
+      </c>
+      <c r="K195" t="n">
+        <v>20</v>
+      </c>
+      <c r="L195" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M195" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N195" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O195" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P195" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q195" t="inlineStr">
+        <is>
+          <t>WeightedRandomSampler equal balance</t>
+        </is>
+      </c>
+      <c r="R195" t="inlineStr">
+        <is>
+          <t>AdamW</t>
+        </is>
+      </c>
+      <c r="S195" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="T195" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="U195" t="n">
+        <v>32</v>
+      </c>
+      <c r="V195" t="n">
+        <v>20</v>
+      </c>
+      <c r="W195" t="inlineStr">
+        <is>
+          <t>CosineAnnealingLR (T_max=20)</t>
+        </is>
+      </c>
+      <c r="X195" t="inlineStr">
+        <is>
+          <t>256x256</t>
+        </is>
+      </c>
+      <c r="Y195" t="inlineStr">
+        <is>
+          <t>HFlip, VFlip, Rotation(15°), ColorJitter(b=0.2,c=0.2), ImageNet norm</t>
+        </is>
+      </c>
+      <c r="Z195" t="n">
+        <v>0.8897</v>
+      </c>
+      <c r="AA195" t="n">
+        <v>0.9863</v>
+      </c>
+      <c r="AB195" t="n">
+        <v>0.9415</v>
+      </c>
+      <c r="AC195" t="n">
+        <v>0.9634</v>
+      </c>
+      <c r="AD195" t="n">
+        <v>0.734</v>
+      </c>
+      <c r="AE195" t="n">
+        <v>0.7419</v>
+      </c>
+      <c r="AF195" t="n">
+        <v>0.738</v>
+      </c>
+      <c r="AG195" t="n">
+        <v>0.5802</v>
+      </c>
+      <c r="AH195" t="n">
+        <v>0.5109</v>
+      </c>
+      <c r="AI195" t="n">
+        <v>0.5434</v>
+      </c>
+      <c r="AJ195" t="n">
+        <v>0.6627</v>
+      </c>
+      <c r="AK195" t="n">
+        <v>0.9322</v>
+      </c>
+      <c r="AL195" t="n">
+        <v>0.7746</v>
+      </c>
+      <c r="AM195" t="n">
+        <v>0.7606000000000001</v>
+      </c>
+      <c r="AN195" t="n">
+        <v>0.9643</v>
+      </c>
+      <c r="AO195" t="n">
+        <v>0.8504</v>
+      </c>
+      <c r="AP195" t="n">
+        <v>0.7739</v>
+      </c>
+      <c r="AQ195" t="n">
+        <v>0.891</v>
+      </c>
+      <c r="AR195" t="n">
+        <v>0.8903</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="n">
+        <v>194</v>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>efficientnet_b4</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>efficientnet_b4</t>
+        </is>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>ImageNet</t>
+        </is>
+      </c>
+      <c r="F196" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G196" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H196" t="inlineStr">
+        <is>
+          <t>Clustered RBC Count</t>
+        </is>
+      </c>
+      <c r="I196" t="n">
+        <v>70</v>
+      </c>
+      <c r="J196" t="n">
+        <v>10</v>
+      </c>
+      <c r="K196" t="n">
+        <v>20</v>
+      </c>
+      <c r="L196" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M196" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N196" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O196" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P196" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q196" t="inlineStr">
+        <is>
+          <t>WeightedRandomSampler equal balance</t>
+        </is>
+      </c>
+      <c r="R196" t="inlineStr">
+        <is>
+          <t>AdamW</t>
+        </is>
+      </c>
+      <c r="S196" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="T196" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="U196" t="n">
+        <v>32</v>
+      </c>
+      <c r="V196" t="n">
+        <v>20</v>
+      </c>
+      <c r="W196" t="inlineStr">
+        <is>
+          <t>CosineAnnealingLR (T_max=20)</t>
+        </is>
+      </c>
+      <c r="X196" t="inlineStr">
+        <is>
+          <t>256x256</t>
+        </is>
+      </c>
+      <c r="Y196" t="inlineStr">
+        <is>
+          <t>HFlip, VFlip, Rotation(15°), ColorJitter(b=0.2,c=0.2), ImageNet norm</t>
+        </is>
+      </c>
+      <c r="Z196" t="n">
+        <v>0.9049</v>
+      </c>
+      <c r="AA196" t="n">
+        <v>0.9845</v>
+      </c>
+      <c r="AB196" t="n">
+        <v>0.9627</v>
+      </c>
+      <c r="AC196" t="n">
+        <v>0.9735</v>
+      </c>
+      <c r="AD196" t="n">
+        <v>0.7772</v>
+      </c>
+      <c r="AE196" t="n">
+        <v>0.7688</v>
+      </c>
+      <c r="AF196" t="n">
+        <v>0.773</v>
+      </c>
+      <c r="AG196" t="n">
+        <v>0.6571</v>
+      </c>
+      <c r="AH196" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AI196" t="n">
+        <v>0.5679</v>
+      </c>
+      <c r="AJ196" t="n">
+        <v>0.7391</v>
+      </c>
+      <c r="AK196" t="n">
+        <v>0.8643999999999999</v>
+      </c>
+      <c r="AL196" t="n">
+        <v>0.7969000000000001</v>
+      </c>
+      <c r="AM196" t="n">
+        <v>0.7365</v>
+      </c>
+      <c r="AN196" t="n">
+        <v>0.9732</v>
+      </c>
+      <c r="AO196" t="n">
+        <v>0.8385</v>
+      </c>
+      <c r="AP196" t="n">
+        <v>0.7899</v>
+      </c>
+      <c r="AQ196" t="n">
+        <v>0.904</v>
+      </c>
+      <c r="AR196" t="n">
+        <v>0.9153</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="n">
+        <v>195</v>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>convnext_tiny</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>convnext_tiny</t>
+        </is>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>ImageNet</t>
+        </is>
+      </c>
+      <c r="F197" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G197" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H197" t="inlineStr">
+        <is>
+          <t>Clustered RBC Count</t>
+        </is>
+      </c>
+      <c r="I197" t="n">
+        <v>70</v>
+      </c>
+      <c r="J197" t="n">
+        <v>10</v>
+      </c>
+      <c r="K197" t="n">
+        <v>20</v>
+      </c>
+      <c r="L197" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M197" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N197" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O197" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P197" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q197" t="inlineStr">
+        <is>
+          <t>WeightedRandomSampler equal balance</t>
+        </is>
+      </c>
+      <c r="R197" t="inlineStr">
+        <is>
+          <t>AdamW</t>
+        </is>
+      </c>
+      <c r="S197" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="T197" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="U197" t="n">
+        <v>32</v>
+      </c>
+      <c r="V197" t="n">
+        <v>20</v>
+      </c>
+      <c r="W197" t="inlineStr">
+        <is>
+          <t>CosineAnnealingLR (T_max=20)</t>
+        </is>
+      </c>
+      <c r="X197" t="inlineStr">
+        <is>
+          <t>256x256</t>
+        </is>
+      </c>
+      <c r="Y197" t="inlineStr">
+        <is>
+          <t>HFlip, VFlip, Rotation(15°), ColorJitter(b=0.2,c=0.2), ImageNet norm</t>
+        </is>
+      </c>
+      <c r="Z197" t="n">
+        <v>0.9368</v>
+      </c>
+      <c r="AA197" t="n">
+        <v>0.9938</v>
+      </c>
+      <c r="AB197" t="n">
+        <v>0.9647</v>
+      </c>
+      <c r="AC197" t="n">
+        <v>0.979</v>
+      </c>
+      <c r="AD197" t="n">
+        <v>0.8778</v>
+      </c>
+      <c r="AE197" t="n">
+        <v>0.8495</v>
+      </c>
+      <c r="AF197" t="n">
+        <v>0.8633999999999999</v>
+      </c>
+      <c r="AG197" t="n">
+        <v>0.729</v>
+      </c>
+      <c r="AH197" t="n">
+        <v>0.8478</v>
+      </c>
+      <c r="AI197" t="n">
+        <v>0.7839</v>
+      </c>
+      <c r="AJ197" t="n">
+        <v>0.8571</v>
+      </c>
+      <c r="AK197" t="n">
+        <v>0.8136</v>
+      </c>
+      <c r="AL197" t="n">
+        <v>0.8348</v>
+      </c>
+      <c r="AM197" t="n">
+        <v>0.8074</v>
+      </c>
+      <c r="AN197" t="n">
+        <v>0.9732</v>
+      </c>
+      <c r="AO197" t="n">
+        <v>0.8826000000000001</v>
+      </c>
+      <c r="AP197" t="n">
+        <v>0.8687</v>
+      </c>
+      <c r="AQ197" t="n">
+        <v>0.9382</v>
+      </c>
+      <c r="AR197" t="n">
+        <v>0.9333</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="n">
+        <v>196</v>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>convnext_base</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>convnext_base</t>
+        </is>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>ImageNet</t>
+        </is>
+      </c>
+      <c r="F198" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G198" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H198" t="inlineStr">
+        <is>
+          <t>Clustered RBC Count</t>
+        </is>
+      </c>
+      <c r="I198" t="n">
+        <v>70</v>
+      </c>
+      <c r="J198" t="n">
+        <v>10</v>
+      </c>
+      <c r="K198" t="n">
+        <v>20</v>
+      </c>
+      <c r="L198" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M198" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N198" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O198" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P198" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q198" t="inlineStr">
+        <is>
+          <t>WeightedRandomSampler equal balance</t>
+        </is>
+      </c>
+      <c r="R198" t="inlineStr">
+        <is>
+          <t>AdamW</t>
+        </is>
+      </c>
+      <c r="S198" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="T198" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="U198" t="n">
+        <v>32</v>
+      </c>
+      <c r="V198" t="n">
+        <v>20</v>
+      </c>
+      <c r="W198" t="inlineStr">
+        <is>
+          <t>CosineAnnealingLR (T_max=20)</t>
+        </is>
+      </c>
+      <c r="X198" t="inlineStr">
+        <is>
+          <t>256x256</t>
+        </is>
+      </c>
+      <c r="Y198" t="inlineStr">
+        <is>
+          <t>HFlip, VFlip, Rotation(15°), ColorJitter(b=0.2,c=0.2), ImageNet norm</t>
+        </is>
+      </c>
+      <c r="Z198" t="n">
+        <v>0.9459</v>
+      </c>
+      <c r="AA198" t="n">
+        <v>0.9918</v>
+      </c>
+      <c r="AB198" t="n">
+        <v>0.9728</v>
+      </c>
+      <c r="AC198" t="n">
+        <v>0.9822</v>
+      </c>
+      <c r="AD198" t="n">
+        <v>0.9314</v>
+      </c>
+      <c r="AE198" t="n">
+        <v>0.8763</v>
+      </c>
+      <c r="AF198" t="n">
+        <v>0.903</v>
+      </c>
+      <c r="AG198" t="n">
+        <v>0.7812</v>
+      </c>
+      <c r="AH198" t="n">
+        <v>0.8152</v>
+      </c>
+      <c r="AI198" t="n">
+        <v>0.7979000000000001</v>
+      </c>
+      <c r="AJ198" t="n">
+        <v>0.803</v>
+      </c>
+      <c r="AK198" t="n">
+        <v>0.8983</v>
+      </c>
+      <c r="AL198" t="n">
+        <v>0.848</v>
+      </c>
+      <c r="AM198" t="n">
+        <v>0.8168</v>
+      </c>
+      <c r="AN198" t="n">
+        <v>0.9554</v>
+      </c>
+      <c r="AO198" t="n">
+        <v>0.8807</v>
+      </c>
+      <c r="AP198" t="n">
+        <v>0.8824</v>
+      </c>
+      <c r="AQ198" t="n">
+        <v>0.9468</v>
+      </c>
+      <c r="AR198" t="n">
+        <v>0.9444</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="n">
+        <v>197</v>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>vit_b16</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>vit_b16</t>
+        </is>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>ImageNet</t>
+        </is>
+      </c>
+      <c r="F199" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G199" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H199" t="inlineStr">
+        <is>
+          <t>Clustered RBC Count</t>
+        </is>
+      </c>
+      <c r="I199" t="n">
+        <v>70</v>
+      </c>
+      <c r="J199" t="n">
+        <v>10</v>
+      </c>
+      <c r="K199" t="n">
+        <v>20</v>
+      </c>
+      <c r="L199" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M199" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N199" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O199" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P199" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q199" t="inlineStr">
+        <is>
+          <t>WeightedRandomSampler equal balance</t>
+        </is>
+      </c>
+      <c r="R199" t="inlineStr">
+        <is>
+          <t>AdamW</t>
+        </is>
+      </c>
+      <c r="S199" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="T199" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="U199" t="n">
+        <v>32</v>
+      </c>
+      <c r="V199" t="n">
+        <v>20</v>
+      </c>
+      <c r="W199" t="inlineStr">
+        <is>
+          <t>CosineAnnealingLR (T_max=20)</t>
+        </is>
+      </c>
+      <c r="X199" t="inlineStr">
+        <is>
+          <t>256x256</t>
+        </is>
+      </c>
+      <c r="Y199" t="inlineStr">
+        <is>
+          <t>HFlip, VFlip, Rotation(15°), ColorJitter(b=0.2,c=0.2), ImageNet norm</t>
+        </is>
+      </c>
+      <c r="Z199" t="n">
+        <v>0.9257</v>
+      </c>
+      <c r="AA199" t="n">
+        <v>0.9897</v>
+      </c>
+      <c r="AB199" t="n">
+        <v>0.9698</v>
+      </c>
+      <c r="AC199" t="n">
+        <v>0.9796</v>
+      </c>
+      <c r="AD199" t="n">
+        <v>0.8678</v>
+      </c>
+      <c r="AE199" t="n">
+        <v>0.8118</v>
+      </c>
+      <c r="AF199" t="n">
+        <v>0.8389</v>
+      </c>
+      <c r="AG199" t="n">
+        <v>0.6966</v>
+      </c>
+      <c r="AH199" t="n">
+        <v>0.6739000000000001</v>
+      </c>
+      <c r="AI199" t="n">
+        <v>0.6851</v>
+      </c>
+      <c r="AJ199" t="n">
+        <v>0.6588000000000001</v>
+      </c>
+      <c r="AK199" t="n">
+        <v>0.9492</v>
+      </c>
+      <c r="AL199" t="n">
+        <v>0.7778</v>
+      </c>
+      <c r="AM199" t="n">
+        <v>0.8512</v>
+      </c>
+      <c r="AN199" t="n">
+        <v>0.9196</v>
+      </c>
+      <c r="AO199" t="n">
+        <v>0.8841</v>
+      </c>
+      <c r="AP199" t="n">
+        <v>0.8331</v>
+      </c>
+      <c r="AQ199" t="n">
+        <v>0.927</v>
+      </c>
+      <c r="AR199" t="n">
+        <v>0.9361</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="R1:Y1"/>

</xml_diff>

<commit_message>
Active Learning Attempt + retraining unclustered RBC count
Trying to setup the cascaded decision tree
</commit_message>
<xml_diff>
--- a/experiment_log.xlsx
+++ b/experiment_log.xlsx
@@ -599,7 +599,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR199"/>
+  <dimension ref="A1:AR224"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -28521,6 +28521,3481 @@
         <v>0.9361</v>
       </c>
     </row>
+    <row r="200">
+      <c r="A200" t="n">
+        <v>198</v>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>default config run</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>convnext_tiny</t>
+        </is>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>ImageNet</t>
+        </is>
+      </c>
+      <c r="F200" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G200" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H200" t="n">
+        <v>12494</v>
+      </c>
+      <c r="I200" t="n">
+        <v>70</v>
+      </c>
+      <c r="J200" t="n">
+        <v>10</v>
+      </c>
+      <c r="K200" t="n">
+        <v>20</v>
+      </c>
+      <c r="L200" t="n">
+        <v>3150</v>
+      </c>
+      <c r="M200" t="n">
+        <v>2421</v>
+      </c>
+      <c r="N200" t="n">
+        <v>807</v>
+      </c>
+      <c r="O200" t="n">
+        <v>807</v>
+      </c>
+      <c r="P200" t="n">
+        <v>807</v>
+      </c>
+      <c r="Q200" t="inlineStr">
+        <is>
+          <t>Per-subclass inverse frequency</t>
+        </is>
+      </c>
+      <c r="R200" t="inlineStr">
+        <is>
+          <t>AdamW</t>
+        </is>
+      </c>
+      <c r="S200" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="T200" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="U200" t="n">
+        <v>32</v>
+      </c>
+      <c r="V200" t="n">
+        <v>20</v>
+      </c>
+      <c r="W200" t="inlineStr">
+        <is>
+          <t>CosineAnnealingLR (T_max=20)</t>
+        </is>
+      </c>
+      <c r="X200" t="inlineStr">
+        <is>
+          <t>256x256</t>
+        </is>
+      </c>
+      <c r="Y200" t="inlineStr">
+        <is>
+          <t>HFlip, VFlip, Rotation(15°), ColorJitter(b=0.2,c=0.2), ImageNet norm</t>
+        </is>
+      </c>
+      <c r="Z200" t="n">
+        <v>0.9268</v>
+      </c>
+      <c r="AA200" t="n">
+        <v>0.8159999999999999</v>
+      </c>
+      <c r="AB200" t="n">
+        <v>0.7865</v>
+      </c>
+      <c r="AC200" t="n">
+        <v>0.801</v>
+      </c>
+      <c r="AD200" t="n">
+        <v>0.9512</v>
+      </c>
+      <c r="AE200" t="n">
+        <v>0.9592000000000001</v>
+      </c>
+      <c r="AF200" t="n">
+        <v>0.9552</v>
+      </c>
+      <c r="AG200" t="n">
+        <v>0.8781</v>
+      </c>
+      <c r="AH200" t="n">
+        <v>0.9263</v>
+      </c>
+      <c r="AI200" t="n">
+        <v>2536</v>
+      </c>
+      <c r="AJ200" t="n">
+        <v>479</v>
+      </c>
+      <c r="AK200" t="n">
+        <v>130</v>
+      </c>
+      <c r="AL200" t="n">
+        <v>108</v>
+      </c>
+      <c r="AM200" t="n">
+        <v>0.9249000000000001</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="n">
+        <v>199</v>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>default config run</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>convnext_tiny</t>
+        </is>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>ImageNet</t>
+        </is>
+      </c>
+      <c r="F201" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G201" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H201" t="n">
+        <v>12494</v>
+      </c>
+      <c r="I201" t="n">
+        <v>70</v>
+      </c>
+      <c r="J201" t="n">
+        <v>10</v>
+      </c>
+      <c r="K201" t="n">
+        <v>20</v>
+      </c>
+      <c r="L201" t="n">
+        <v>3150</v>
+      </c>
+      <c r="M201" t="n">
+        <v>2421</v>
+      </c>
+      <c r="N201" t="n">
+        <v>807</v>
+      </c>
+      <c r="O201" t="n">
+        <v>807</v>
+      </c>
+      <c r="P201" t="n">
+        <v>807</v>
+      </c>
+      <c r="Q201" t="inlineStr">
+        <is>
+          <t>Per-subclass inverse frequency</t>
+        </is>
+      </c>
+      <c r="R201" t="inlineStr">
+        <is>
+          <t>AdamW</t>
+        </is>
+      </c>
+      <c r="S201" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="T201" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="U201" t="n">
+        <v>32</v>
+      </c>
+      <c r="V201" t="n">
+        <v>20</v>
+      </c>
+      <c r="W201" t="inlineStr">
+        <is>
+          <t>CosineAnnealingLR (T_max=20)</t>
+        </is>
+      </c>
+      <c r="X201" t="inlineStr">
+        <is>
+          <t>256x256</t>
+        </is>
+      </c>
+      <c r="Y201" t="inlineStr">
+        <is>
+          <t>HFlip, VFlip, Rotation(15°), ColorJitter(b=0.2,c=0.2), ImageNet norm</t>
+        </is>
+      </c>
+      <c r="Z201" t="n">
+        <v>0.9127</v>
+      </c>
+      <c r="AA201" t="n">
+        <v>0.7651</v>
+      </c>
+      <c r="AB201" t="n">
+        <v>0.7701</v>
+      </c>
+      <c r="AC201" t="n">
+        <v>0.7675999999999999</v>
+      </c>
+      <c r="AD201" t="n">
+        <v>0.947</v>
+      </c>
+      <c r="AE201" t="n">
+        <v>0.9455</v>
+      </c>
+      <c r="AF201" t="n">
+        <v>0.9463</v>
+      </c>
+      <c r="AG201" t="n">
+        <v>0.8569</v>
+      </c>
+      <c r="AH201" t="n">
+        <v>0.9127999999999999</v>
+      </c>
+      <c r="AI201" t="n">
+        <v>2500</v>
+      </c>
+      <c r="AJ201" t="n">
+        <v>469</v>
+      </c>
+      <c r="AK201" t="n">
+        <v>140</v>
+      </c>
+      <c r="AL201" t="n">
+        <v>144</v>
+      </c>
+      <c r="AM201" t="n">
+        <v>0.9188</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="n">
+        <v>200</v>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>2450 each class</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>convnext_tiny</t>
+        </is>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>ImageNet</t>
+        </is>
+      </c>
+      <c r="F202" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G202" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H202" t="n">
+        <v>12494</v>
+      </c>
+      <c r="I202" t="n">
+        <v>70</v>
+      </c>
+      <c r="J202" t="n">
+        <v>10</v>
+      </c>
+      <c r="K202" t="n">
+        <v>20</v>
+      </c>
+      <c r="L202" t="n">
+        <v>2450</v>
+      </c>
+      <c r="M202" t="n">
+        <v>2450</v>
+      </c>
+      <c r="N202" t="n">
+        <v>816</v>
+      </c>
+      <c r="O202" t="n">
+        <v>816</v>
+      </c>
+      <c r="P202" t="n">
+        <v>818</v>
+      </c>
+      <c r="Q202" t="inlineStr">
+        <is>
+          <t>Per-subclass inverse frequency</t>
+        </is>
+      </c>
+      <c r="R202" t="inlineStr">
+        <is>
+          <t>AdamW</t>
+        </is>
+      </c>
+      <c r="S202" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="T202" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="U202" t="n">
+        <v>32</v>
+      </c>
+      <c r="V202" t="n">
+        <v>20</v>
+      </c>
+      <c r="W202" t="inlineStr">
+        <is>
+          <t>CosineAnnealingLR (T_max=20)</t>
+        </is>
+      </c>
+      <c r="X202" t="inlineStr">
+        <is>
+          <t>256x256</t>
+        </is>
+      </c>
+      <c r="Y202" t="inlineStr">
+        <is>
+          <t>HFlip, VFlip, Rotation(15°), ColorJitter(b=0.2,c=0.2), ImageNet norm</t>
+        </is>
+      </c>
+      <c r="Z202" t="n">
+        <v>0.9247</v>
+      </c>
+      <c r="AA202" t="n">
+        <v>0.8023</v>
+      </c>
+      <c r="AB202" t="n">
+        <v>0.7931</v>
+      </c>
+      <c r="AC202" t="n">
+        <v>0.7977</v>
+      </c>
+      <c r="AD202" t="n">
+        <v>0.9525</v>
+      </c>
+      <c r="AE202" t="n">
+        <v>0.955</v>
+      </c>
+      <c r="AF202" t="n">
+        <v>0.9537</v>
+      </c>
+      <c r="AG202" t="n">
+        <v>0.8757</v>
+      </c>
+      <c r="AH202" t="n">
+        <v>0.9245</v>
+      </c>
+      <c r="AI202" t="n">
+        <v>2525</v>
+      </c>
+      <c r="AJ202" t="n">
+        <v>483</v>
+      </c>
+      <c r="AK202" t="n">
+        <v>126</v>
+      </c>
+      <c r="AL202" t="n">
+        <v>119</v>
+      </c>
+      <c r="AM202" t="n">
+        <v>0.9249000000000001</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="n">
+        <v>201</v>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>Stage1_fixed_split</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>convnext_tiny</t>
+        </is>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>ImageNet</t>
+        </is>
+      </c>
+      <c r="F203" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G203" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H203" t="n">
+        <v>12494</v>
+      </c>
+      <c r="I203" t="n">
+        <v>70</v>
+      </c>
+      <c r="J203" t="n">
+        <v>10</v>
+      </c>
+      <c r="K203" t="n">
+        <v>20</v>
+      </c>
+      <c r="L203" t="n">
+        <v>2450</v>
+      </c>
+      <c r="M203" t="n">
+        <v>2450</v>
+      </c>
+      <c r="N203" t="n">
+        <v>816</v>
+      </c>
+      <c r="O203" t="n">
+        <v>816</v>
+      </c>
+      <c r="P203" t="n">
+        <v>818</v>
+      </c>
+      <c r="Q203" t="inlineStr">
+        <is>
+          <t>Per-subclass inverse frequency</t>
+        </is>
+      </c>
+      <c r="R203" t="inlineStr">
+        <is>
+          <t>AdamW</t>
+        </is>
+      </c>
+      <c r="S203" t="n">
+        <v>1e-05</v>
+      </c>
+      <c r="T203" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="U203" t="n">
+        <v>32</v>
+      </c>
+      <c r="V203" t="n">
+        <v>30</v>
+      </c>
+      <c r="W203" t="inlineStr">
+        <is>
+          <t>CosineAnnealingLR (T_max=30)</t>
+        </is>
+      </c>
+      <c r="X203" t="inlineStr">
+        <is>
+          <t>256x256</t>
+        </is>
+      </c>
+      <c r="Y203" t="inlineStr">
+        <is>
+          <t>HFlip, VFlip, Rotation(15°), ColorJitter(b=0.2,c=0.2), ImageNet norm</t>
+        </is>
+      </c>
+      <c r="Z203" t="n">
+        <v>0.9046999999999999</v>
+      </c>
+      <c r="AA203" t="n">
+        <v>0.8211000000000001</v>
+      </c>
+      <c r="AB203" t="n">
+        <v>0.6266</v>
+      </c>
+      <c r="AC203" t="n">
+        <v>0.7108</v>
+      </c>
+      <c r="AD203" t="n">
+        <v>0.9186</v>
+      </c>
+      <c r="AE203" t="n">
+        <v>0.9686</v>
+      </c>
+      <c r="AF203" t="n">
+        <v>0.9429</v>
+      </c>
+      <c r="AG203" t="n">
+        <v>0.8269</v>
+      </c>
+      <c r="AH203" t="n">
+        <v>0.8995</v>
+      </c>
+      <c r="AI203" t="n">
+        <v>2561</v>
+      </c>
+      <c r="AJ203" t="n">
+        <v>381</v>
+      </c>
+      <c r="AK203" t="n">
+        <v>227</v>
+      </c>
+      <c r="AL203" t="n">
+        <v>83</v>
+      </c>
+      <c r="AM203" t="n">
+        <v>0.9096</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="n">
+        <v>202</v>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>ActiveLearningRound</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>convnext_tiny</t>
+        </is>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>ImageNet</t>
+        </is>
+      </c>
+      <c r="F204" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G204" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H204" t="n">
+        <v>12494</v>
+      </c>
+      <c r="I204" t="n">
+        <v>70</v>
+      </c>
+      <c r="J204" t="n">
+        <v>10</v>
+      </c>
+      <c r="K204" t="n">
+        <v>20</v>
+      </c>
+      <c r="L204" t="n">
+        <v>2450</v>
+      </c>
+      <c r="M204" t="n">
+        <v>2450</v>
+      </c>
+      <c r="N204" t="n">
+        <v>816</v>
+      </c>
+      <c r="O204" t="n">
+        <v>816</v>
+      </c>
+      <c r="P204" t="n">
+        <v>818</v>
+      </c>
+      <c r="Q204" t="inlineStr">
+        <is>
+          <t>Per-subclass inverse frequency</t>
+        </is>
+      </c>
+      <c r="R204" t="inlineStr">
+        <is>
+          <t>AdamW</t>
+        </is>
+      </c>
+      <c r="S204" t="n">
+        <v>1e-05</v>
+      </c>
+      <c r="T204" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="U204" t="n">
+        <v>32</v>
+      </c>
+      <c r="V204" t="n">
+        <v>30</v>
+      </c>
+      <c r="W204" t="inlineStr">
+        <is>
+          <t>CosineAnnealingLR (T_max=30)</t>
+        </is>
+      </c>
+      <c r="X204" t="inlineStr">
+        <is>
+          <t>256x256</t>
+        </is>
+      </c>
+      <c r="Y204" t="inlineStr">
+        <is>
+          <t>HFlip, VFlip, Rotation(15°), ColorJitter(b=0.2,c=0.2), ImageNet norm</t>
+        </is>
+      </c>
+      <c r="Z204" t="n">
+        <v>0.9053</v>
+      </c>
+      <c r="AA204" t="n">
+        <v>0.6963</v>
+      </c>
+      <c r="AB204" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="AC204" t="n">
+        <v>0.7755</v>
+      </c>
+      <c r="AD204" t="n">
+        <v>0.9695</v>
+      </c>
+      <c r="AE204" t="n">
+        <v>0.9123</v>
+      </c>
+      <c r="AF204" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="AG204" t="n">
+        <v>0.8577</v>
+      </c>
+      <c r="AH204" t="n">
+        <v>0.9092</v>
+      </c>
+      <c r="AI204" t="n">
+        <v>2412</v>
+      </c>
+      <c r="AJ204" t="n">
+        <v>532</v>
+      </c>
+      <c r="AK204" t="n">
+        <v>76</v>
+      </c>
+      <c r="AL204" t="n">
+        <v>232</v>
+      </c>
+      <c r="AM204" t="n">
+        <v>0.9034</v>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="n">
+        <v>203</v>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>ActiveLearningRound</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>convnext_tiny</t>
+        </is>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>ImageNet</t>
+        </is>
+      </c>
+      <c r="F205" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G205" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H205" t="n">
+        <v>12494</v>
+      </c>
+      <c r="I205" t="n">
+        <v>70</v>
+      </c>
+      <c r="J205" t="n">
+        <v>10</v>
+      </c>
+      <c r="K205" t="n">
+        <v>20</v>
+      </c>
+      <c r="L205" t="n">
+        <v>2450</v>
+      </c>
+      <c r="M205" t="n">
+        <v>2450</v>
+      </c>
+      <c r="N205" t="n">
+        <v>816</v>
+      </c>
+      <c r="O205" t="n">
+        <v>816</v>
+      </c>
+      <c r="P205" t="n">
+        <v>818</v>
+      </c>
+      <c r="Q205" t="inlineStr">
+        <is>
+          <t>Per-subclass inverse frequency</t>
+        </is>
+      </c>
+      <c r="R205" t="inlineStr">
+        <is>
+          <t>AdamW</t>
+        </is>
+      </c>
+      <c r="S205" t="n">
+        <v>1e-05</v>
+      </c>
+      <c r="T205" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="U205" t="n">
+        <v>32</v>
+      </c>
+      <c r="V205" t="n">
+        <v>30</v>
+      </c>
+      <c r="W205" t="inlineStr">
+        <is>
+          <t>CosineAnnealingLR (T_max=30)</t>
+        </is>
+      </c>
+      <c r="X205" t="inlineStr">
+        <is>
+          <t>256x256</t>
+        </is>
+      </c>
+      <c r="Y205" t="inlineStr">
+        <is>
+          <t>HFlip, VFlip, Rotation(15°), ColorJitter(b=0.2,c=0.2), ImageNet norm</t>
+        </is>
+      </c>
+      <c r="Z205" t="n">
+        <v>0.9044</v>
+      </c>
+      <c r="AA205" t="n">
+        <v>0.7106</v>
+      </c>
+      <c r="AB205" t="n">
+        <v>0.824</v>
+      </c>
+      <c r="AC205" t="n">
+        <v>0.7631</v>
+      </c>
+      <c r="AD205" t="n">
+        <v>0.958</v>
+      </c>
+      <c r="AE205" t="n">
+        <v>0.9228</v>
+      </c>
+      <c r="AF205" t="n">
+        <v>0.9401</v>
+      </c>
+      <c r="AG205" t="n">
+        <v>0.8516</v>
+      </c>
+      <c r="AH205" t="n">
+        <v>0.907</v>
+      </c>
+      <c r="AI205" t="n">
+        <v>2440</v>
+      </c>
+      <c r="AJ205" t="n">
+        <v>501</v>
+      </c>
+      <c r="AK205" t="n">
+        <v>107</v>
+      </c>
+      <c r="AL205" t="n">
+        <v>204</v>
+      </c>
+      <c r="AM205" t="n">
+        <v>0.8979</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="n">
+        <v>204</v>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>ActiveLearningRound</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>convnext_tiny</t>
+        </is>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>ImageNet</t>
+        </is>
+      </c>
+      <c r="F206" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G206" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H206" t="n">
+        <v>12494</v>
+      </c>
+      <c r="I206" t="n">
+        <v>70</v>
+      </c>
+      <c r="J206" t="n">
+        <v>10</v>
+      </c>
+      <c r="K206" t="n">
+        <v>20</v>
+      </c>
+      <c r="L206" t="n">
+        <v>2450</v>
+      </c>
+      <c r="M206" t="n">
+        <v>2450</v>
+      </c>
+      <c r="N206" t="n">
+        <v>816</v>
+      </c>
+      <c r="O206" t="n">
+        <v>816</v>
+      </c>
+      <c r="P206" t="n">
+        <v>818</v>
+      </c>
+      <c r="Q206" t="inlineStr">
+        <is>
+          <t>Per-subclass inverse frequency</t>
+        </is>
+      </c>
+      <c r="R206" t="inlineStr">
+        <is>
+          <t>AdamW</t>
+        </is>
+      </c>
+      <c r="S206" t="n">
+        <v>1e-05</v>
+      </c>
+      <c r="T206" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="U206" t="n">
+        <v>32</v>
+      </c>
+      <c r="V206" t="n">
+        <v>30</v>
+      </c>
+      <c r="W206" t="inlineStr">
+        <is>
+          <t>CosineAnnealingLR (T_max=30)</t>
+        </is>
+      </c>
+      <c r="X206" t="inlineStr">
+        <is>
+          <t>256x256</t>
+        </is>
+      </c>
+      <c r="Y206" t="inlineStr">
+        <is>
+          <t>HFlip, VFlip, Rotation(15°), ColorJitter(b=0.2,c=0.2), ImageNet norm</t>
+        </is>
+      </c>
+      <c r="Z206" t="n">
+        <v>0.9124</v>
+      </c>
+      <c r="AA206" t="n">
+        <v>0.6962</v>
+      </c>
+      <c r="AB206" t="n">
+        <v>0.9024</v>
+      </c>
+      <c r="AC206" t="n">
+        <v>0.786</v>
+      </c>
+      <c r="AD206" t="n">
+        <v>0.9774</v>
+      </c>
+      <c r="AE206" t="n">
+        <v>0.9145</v>
+      </c>
+      <c r="AF206" t="n">
+        <v>0.9449</v>
+      </c>
+      <c r="AG206" t="n">
+        <v>0.8655</v>
+      </c>
+      <c r="AH206" t="n">
+        <v>0.9166</v>
+      </c>
+      <c r="AI206" t="n">
+        <v>2418</v>
+      </c>
+      <c r="AJ206" t="n">
+        <v>518</v>
+      </c>
+      <c r="AK206" t="n">
+        <v>56</v>
+      </c>
+      <c r="AL206" t="n">
+        <v>226</v>
+      </c>
+      <c r="AM206" t="n">
+        <v>0.9216</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="n">
+        <v>205</v>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>default config run</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>resnet34</t>
+        </is>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>ImageNet</t>
+        </is>
+      </c>
+      <c r="F207" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G207" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H207" t="n">
+        <v>12494</v>
+      </c>
+      <c r="I207" t="n">
+        <v>70</v>
+      </c>
+      <c r="J207" t="n">
+        <v>10</v>
+      </c>
+      <c r="K207" t="n">
+        <v>20</v>
+      </c>
+      <c r="L207" t="n">
+        <v>2200</v>
+      </c>
+      <c r="M207" t="n">
+        <v>2421</v>
+      </c>
+      <c r="N207" t="n">
+        <v>807</v>
+      </c>
+      <c r="O207" t="n">
+        <v>807</v>
+      </c>
+      <c r="P207" t="n">
+        <v>807</v>
+      </c>
+      <c r="Q207" t="inlineStr">
+        <is>
+          <t>Per-subclass inverse frequency</t>
+        </is>
+      </c>
+      <c r="R207" t="inlineStr">
+        <is>
+          <t>AdamW</t>
+        </is>
+      </c>
+      <c r="S207" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="T207" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="U207" t="n">
+        <v>32</v>
+      </c>
+      <c r="V207" t="n">
+        <v>20</v>
+      </c>
+      <c r="W207" t="inlineStr">
+        <is>
+          <t>CosineAnnealingLR (T_max=20)</t>
+        </is>
+      </c>
+      <c r="X207" t="inlineStr">
+        <is>
+          <t>256x256</t>
+        </is>
+      </c>
+      <c r="Y207" t="inlineStr">
+        <is>
+          <t>HFlip, VFlip, Rotation(15°), ColorJitter(b=0.2,c=0.2), ImageNet norm</t>
+        </is>
+      </c>
+      <c r="Z207" t="n">
+        <v>0.9099</v>
+      </c>
+      <c r="AA207" t="n">
+        <v>0.7625</v>
+      </c>
+      <c r="AB207" t="n">
+        <v>0.7173</v>
+      </c>
+      <c r="AC207" t="n">
+        <v>0.7392</v>
+      </c>
+      <c r="AD207" t="n">
+        <v>0.9395</v>
+      </c>
+      <c r="AE207" t="n">
+        <v>0.9516</v>
+      </c>
+      <c r="AF207" t="n">
+        <v>0.9455</v>
+      </c>
+      <c r="AG207" t="n">
+        <v>0.8424</v>
+      </c>
+      <c r="AH207" t="n">
+        <v>0.9088000000000001</v>
+      </c>
+      <c r="AI207" t="n">
+        <v>2517</v>
+      </c>
+      <c r="AJ207" t="n">
+        <v>411</v>
+      </c>
+      <c r="AK207" t="n">
+        <v>162</v>
+      </c>
+      <c r="AL207" t="n">
+        <v>128</v>
+      </c>
+      <c r="AM207" t="n">
+        <v>0.9036</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="n">
+        <v>206</v>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>resnet34 baseline kfold | fold 1/5</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>resnet34</t>
+        </is>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>ImageNet</t>
+        </is>
+      </c>
+      <c r="F208" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G208" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H208" t="n">
+        <v>12494</v>
+      </c>
+      <c r="I208" t="n">
+        <v>70</v>
+      </c>
+      <c r="J208" t="n">
+        <v>10</v>
+      </c>
+      <c r="K208" t="n">
+        <v>20</v>
+      </c>
+      <c r="L208" t="n">
+        <v>2200</v>
+      </c>
+      <c r="M208" t="n">
+        <v>2421</v>
+      </c>
+      <c r="N208" t="n">
+        <v>807</v>
+      </c>
+      <c r="O208" t="n">
+        <v>807</v>
+      </c>
+      <c r="P208" t="n">
+        <v>807</v>
+      </c>
+      <c r="Q208" t="inlineStr">
+        <is>
+          <t>Per-subclass inverse frequency</t>
+        </is>
+      </c>
+      <c r="R208" t="inlineStr">
+        <is>
+          <t>AdamW</t>
+        </is>
+      </c>
+      <c r="S208" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="T208" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="U208" t="n">
+        <v>32</v>
+      </c>
+      <c r="V208" t="n">
+        <v>20</v>
+      </c>
+      <c r="W208" t="inlineStr">
+        <is>
+          <t>CosineAnnealingLR (T_max=20)</t>
+        </is>
+      </c>
+      <c r="X208" t="inlineStr">
+        <is>
+          <t>256x256</t>
+        </is>
+      </c>
+      <c r="Y208" t="inlineStr">
+        <is>
+          <t>HFlip, VFlip, Rotation(15°), ColorJitter(b=0.2,c=0.2), ImageNet norm</t>
+        </is>
+      </c>
+      <c r="Z208" t="n">
+        <v>0.9034</v>
+      </c>
+      <c r="AA208" t="n">
+        <v>0.6938</v>
+      </c>
+      <c r="AB208" t="n">
+        <v>0.8185</v>
+      </c>
+      <c r="AC208" t="n">
+        <v>0.751</v>
+      </c>
+      <c r="AD208" t="n">
+        <v>0.9591</v>
+      </c>
+      <c r="AE208" t="n">
+        <v>0.9217</v>
+      </c>
+      <c r="AF208" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="AG208" t="n">
+        <v>0.8455</v>
+      </c>
+      <c r="AH208" t="n">
+        <v>0.9064</v>
+      </c>
+      <c r="AI208" t="n">
+        <v>2438</v>
+      </c>
+      <c r="AJ208" t="n">
+        <v>469</v>
+      </c>
+      <c r="AK208" t="n">
+        <v>104</v>
+      </c>
+      <c r="AL208" t="n">
+        <v>207</v>
+      </c>
+      <c r="AM208" t="n">
+        <v>0.8999</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="n">
+        <v>207</v>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>resnet34 baseline kfold | fold 2/5</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>resnet34</t>
+        </is>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>ImageNet</t>
+        </is>
+      </c>
+      <c r="F209" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G209" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H209" t="n">
+        <v>12494</v>
+      </c>
+      <c r="I209" t="n">
+        <v>70</v>
+      </c>
+      <c r="J209" t="n">
+        <v>10</v>
+      </c>
+      <c r="K209" t="n">
+        <v>20</v>
+      </c>
+      <c r="L209" t="n">
+        <v>2200</v>
+      </c>
+      <c r="M209" t="n">
+        <v>2421</v>
+      </c>
+      <c r="N209" t="n">
+        <v>807</v>
+      </c>
+      <c r="O209" t="n">
+        <v>807</v>
+      </c>
+      <c r="P209" t="n">
+        <v>807</v>
+      </c>
+      <c r="Q209" t="inlineStr">
+        <is>
+          <t>Per-subclass inverse frequency</t>
+        </is>
+      </c>
+      <c r="R209" t="inlineStr">
+        <is>
+          <t>AdamW</t>
+        </is>
+      </c>
+      <c r="S209" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="T209" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="U209" t="n">
+        <v>32</v>
+      </c>
+      <c r="V209" t="n">
+        <v>20</v>
+      </c>
+      <c r="W209" t="inlineStr">
+        <is>
+          <t>CosineAnnealingLR (T_max=20)</t>
+        </is>
+      </c>
+      <c r="X209" t="inlineStr">
+        <is>
+          <t>256x256</t>
+        </is>
+      </c>
+      <c r="Y209" t="inlineStr">
+        <is>
+          <t>HFlip, VFlip, Rotation(15°), ColorJitter(b=0.2,c=0.2), ImageNet norm</t>
+        </is>
+      </c>
+      <c r="Z209" t="n">
+        <v>0.9195</v>
+      </c>
+      <c r="AA209" t="n">
+        <v>0.7476</v>
+      </c>
+      <c r="AB209" t="n">
+        <v>0.8272</v>
+      </c>
+      <c r="AC209" t="n">
+        <v>0.7854</v>
+      </c>
+      <c r="AD209" t="n">
+        <v>0.9617</v>
+      </c>
+      <c r="AE209" t="n">
+        <v>0.9395</v>
+      </c>
+      <c r="AF209" t="n">
+        <v>0.9505</v>
+      </c>
+      <c r="AG209" t="n">
+        <v>0.8679</v>
+      </c>
+      <c r="AH209" t="n">
+        <v>0.9211</v>
+      </c>
+      <c r="AI209" t="n">
+        <v>2485</v>
+      </c>
+      <c r="AJ209" t="n">
+        <v>474</v>
+      </c>
+      <c r="AK209" t="n">
+        <v>99</v>
+      </c>
+      <c r="AL209" t="n">
+        <v>160</v>
+      </c>
+      <c r="AM209" t="n">
+        <v>0.921</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="n">
+        <v>208</v>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>convnext_tiny target=1500</t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>convnext_tiny</t>
+        </is>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>ImageNet</t>
+        </is>
+      </c>
+      <c r="F210" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G210" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H210" t="n">
+        <v>12494</v>
+      </c>
+      <c r="I210" t="n">
+        <v>70</v>
+      </c>
+      <c r="J210" t="n">
+        <v>10</v>
+      </c>
+      <c r="K210" t="n">
+        <v>20</v>
+      </c>
+      <c r="L210" t="n">
+        <v>1900</v>
+      </c>
+      <c r="M210" t="n">
+        <v>1500</v>
+      </c>
+      <c r="N210" t="n">
+        <v>500</v>
+      </c>
+      <c r="O210" t="n">
+        <v>500</v>
+      </c>
+      <c r="P210" t="n">
+        <v>500</v>
+      </c>
+      <c r="Q210" t="inlineStr">
+        <is>
+          <t>Per-subclass inverse frequency</t>
+        </is>
+      </c>
+      <c r="R210" t="inlineStr">
+        <is>
+          <t>AdamW</t>
+        </is>
+      </c>
+      <c r="S210" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="T210" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="U210" t="n">
+        <v>32</v>
+      </c>
+      <c r="V210" t="n">
+        <v>20</v>
+      </c>
+      <c r="W210" t="inlineStr">
+        <is>
+          <t>CosineAnnealingLR (T_max=20)</t>
+        </is>
+      </c>
+      <c r="X210" t="inlineStr">
+        <is>
+          <t>256x256</t>
+        </is>
+      </c>
+      <c r="Y210" t="inlineStr">
+        <is>
+          <t>HFlip, VFlip, Rotation(15°), ColorJitter(b=0.2,c=0.2), ImageNet norm</t>
+        </is>
+      </c>
+      <c r="Z210" t="n">
+        <v>0.9164</v>
+      </c>
+      <c r="AA210" t="n">
+        <v>0.7249</v>
+      </c>
+      <c r="AB210" t="n">
+        <v>0.8551</v>
+      </c>
+      <c r="AC210" t="n">
+        <v>0.7846</v>
+      </c>
+      <c r="AD210" t="n">
+        <v>0.9673</v>
+      </c>
+      <c r="AE210" t="n">
+        <v>0.9297</v>
+      </c>
+      <c r="AF210" t="n">
+        <v>0.9481000000000001</v>
+      </c>
+      <c r="AG210" t="n">
+        <v>0.8663999999999999</v>
+      </c>
+      <c r="AH210" t="n">
+        <v>0.919</v>
+      </c>
+      <c r="AI210" t="n">
+        <v>2459</v>
+      </c>
+      <c r="AJ210" t="n">
+        <v>490</v>
+      </c>
+      <c r="AK210" t="n">
+        <v>83</v>
+      </c>
+      <c r="AL210" t="n">
+        <v>186</v>
+      </c>
+      <c r="AM210" t="n">
+        <v>0.916</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="n">
+        <v>209</v>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>resnet34 baseline kfold | fold 1/5</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>resnet34</t>
+        </is>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>ImageNet</t>
+        </is>
+      </c>
+      <c r="F211" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G211" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H211" t="n">
+        <v>12494</v>
+      </c>
+      <c r="I211" t="n">
+        <v>70</v>
+      </c>
+      <c r="J211" t="n">
+        <v>10</v>
+      </c>
+      <c r="K211" t="n">
+        <v>20</v>
+      </c>
+      <c r="L211" t="n">
+        <v>2200</v>
+      </c>
+      <c r="M211" t="n">
+        <v>2421</v>
+      </c>
+      <c r="N211" t="n">
+        <v>807</v>
+      </c>
+      <c r="O211" t="n">
+        <v>807</v>
+      </c>
+      <c r="P211" t="n">
+        <v>807</v>
+      </c>
+      <c r="Q211" t="inlineStr">
+        <is>
+          <t>Per-subclass inverse frequency</t>
+        </is>
+      </c>
+      <c r="R211" t="inlineStr">
+        <is>
+          <t>AdamW</t>
+        </is>
+      </c>
+      <c r="S211" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="T211" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="U211" t="n">
+        <v>32</v>
+      </c>
+      <c r="V211" t="n">
+        <v>20</v>
+      </c>
+      <c r="W211" t="inlineStr">
+        <is>
+          <t>CosineAnnealingLR (T_max=20)</t>
+        </is>
+      </c>
+      <c r="X211" t="inlineStr">
+        <is>
+          <t>256x256</t>
+        </is>
+      </c>
+      <c r="Y211" t="inlineStr">
+        <is>
+          <t>HFlip, VFlip, Rotation(15°), ColorJitter(b=0.2,c=0.2), ImageNet norm</t>
+        </is>
+      </c>
+      <c r="Z211" t="n">
+        <v>0.9089</v>
+      </c>
+      <c r="AA211" t="n">
+        <v>0.6966</v>
+      </c>
+      <c r="AB211" t="n">
+        <v>0.8656</v>
+      </c>
+      <c r="AC211" t="n">
+        <v>0.772</v>
+      </c>
+      <c r="AD211" t="n">
+        <v>0.9693000000000001</v>
+      </c>
+      <c r="AE211" t="n">
+        <v>0.9183</v>
+      </c>
+      <c r="AF211" t="n">
+        <v>0.9431</v>
+      </c>
+      <c r="AG211" t="n">
+        <v>0.8576</v>
+      </c>
+      <c r="AH211" t="n">
+        <v>0.9126</v>
+      </c>
+      <c r="AI211" t="n">
+        <v>2429</v>
+      </c>
+      <c r="AJ211" t="n">
+        <v>496</v>
+      </c>
+      <c r="AK211" t="n">
+        <v>77</v>
+      </c>
+      <c r="AL211" t="n">
+        <v>216</v>
+      </c>
+      <c r="AM211" t="n">
+        <v>0.9136</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="n">
+        <v>210</v>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>convnext_tiny target=1500</t>
+        </is>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>convnext_tiny</t>
+        </is>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>ImageNet</t>
+        </is>
+      </c>
+      <c r="F212" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G212" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H212" t="n">
+        <v>12494</v>
+      </c>
+      <c r="I212" t="n">
+        <v>70</v>
+      </c>
+      <c r="J212" t="n">
+        <v>10</v>
+      </c>
+      <c r="K212" t="n">
+        <v>20</v>
+      </c>
+      <c r="L212" t="n">
+        <v>1900</v>
+      </c>
+      <c r="M212" t="n">
+        <v>1500</v>
+      </c>
+      <c r="N212" t="n">
+        <v>500</v>
+      </c>
+      <c r="O212" t="n">
+        <v>500</v>
+      </c>
+      <c r="P212" t="n">
+        <v>500</v>
+      </c>
+      <c r="Q212" t="inlineStr">
+        <is>
+          <t>Per-subclass inverse frequency</t>
+        </is>
+      </c>
+      <c r="R212" t="inlineStr">
+        <is>
+          <t>AdamW</t>
+        </is>
+      </c>
+      <c r="S212" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="T212" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="U212" t="n">
+        <v>32</v>
+      </c>
+      <c r="V212" t="n">
+        <v>20</v>
+      </c>
+      <c r="W212" t="inlineStr">
+        <is>
+          <t>CosineAnnealingLR (T_max=20)</t>
+        </is>
+      </c>
+      <c r="X212" t="inlineStr">
+        <is>
+          <t>256x256</t>
+        </is>
+      </c>
+      <c r="Y212" t="inlineStr">
+        <is>
+          <t>HFlip, VFlip, Rotation(15°), ColorJitter(b=0.2,c=0.2), ImageNet norm</t>
+        </is>
+      </c>
+      <c r="Z212" t="n">
+        <v>0.9152</v>
+      </c>
+      <c r="AA212" t="n">
+        <v>0.7155</v>
+      </c>
+      <c r="AB212" t="n">
+        <v>0.8691</v>
+      </c>
+      <c r="AC212" t="n">
+        <v>0.7849</v>
+      </c>
+      <c r="AD212" t="n">
+        <v>0.9703000000000001</v>
+      </c>
+      <c r="AE212" t="n">
+        <v>0.9251</v>
+      </c>
+      <c r="AF212" t="n">
+        <v>0.9472</v>
+      </c>
+      <c r="AG212" t="n">
+        <v>0.866</v>
+      </c>
+      <c r="AH212" t="n">
+        <v>0.9183</v>
+      </c>
+      <c r="AI212" t="n">
+        <v>2447</v>
+      </c>
+      <c r="AJ212" t="n">
+        <v>498</v>
+      </c>
+      <c r="AK212" t="n">
+        <v>75</v>
+      </c>
+      <c r="AL212" t="n">
+        <v>198</v>
+      </c>
+      <c r="AM212" t="n">
+        <v>0.9147999999999999</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="n">
+        <v>211</v>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>resnet34 baseline kfold | fold 2/5</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>resnet34</t>
+        </is>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>ImageNet</t>
+        </is>
+      </c>
+      <c r="F213" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G213" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H213" t="n">
+        <v>12494</v>
+      </c>
+      <c r="I213" t="n">
+        <v>70</v>
+      </c>
+      <c r="J213" t="n">
+        <v>10</v>
+      </c>
+      <c r="K213" t="n">
+        <v>20</v>
+      </c>
+      <c r="L213" t="n">
+        <v>2200</v>
+      </c>
+      <c r="M213" t="n">
+        <v>2421</v>
+      </c>
+      <c r="N213" t="n">
+        <v>807</v>
+      </c>
+      <c r="O213" t="n">
+        <v>807</v>
+      </c>
+      <c r="P213" t="n">
+        <v>807</v>
+      </c>
+      <c r="Q213" t="inlineStr">
+        <is>
+          <t>Per-subclass inverse frequency</t>
+        </is>
+      </c>
+      <c r="R213" t="inlineStr">
+        <is>
+          <t>AdamW</t>
+        </is>
+      </c>
+      <c r="S213" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="T213" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="U213" t="n">
+        <v>32</v>
+      </c>
+      <c r="V213" t="n">
+        <v>20</v>
+      </c>
+      <c r="W213" t="inlineStr">
+        <is>
+          <t>CosineAnnealingLR (T_max=20)</t>
+        </is>
+      </c>
+      <c r="X213" t="inlineStr">
+        <is>
+          <t>256x256</t>
+        </is>
+      </c>
+      <c r="Y213" t="inlineStr">
+        <is>
+          <t>HFlip, VFlip, Rotation(15°), ColorJitter(b=0.2,c=0.2), ImageNet norm</t>
+        </is>
+      </c>
+      <c r="Z213" t="n">
+        <v>0.9145</v>
+      </c>
+      <c r="AA213" t="n">
+        <v>0.7217</v>
+      </c>
+      <c r="AB213" t="n">
+        <v>0.8464</v>
+      </c>
+      <c r="AC213" t="n">
+        <v>0.7791</v>
+      </c>
+      <c r="AD213" t="n">
+        <v>0.9654</v>
+      </c>
+      <c r="AE213" t="n">
+        <v>0.9293</v>
+      </c>
+      <c r="AF213" t="n">
+        <v>0.947</v>
+      </c>
+      <c r="AG213" t="n">
+        <v>0.8631</v>
+      </c>
+      <c r="AH213" t="n">
+        <v>0.9171</v>
+      </c>
+      <c r="AI213" t="n">
+        <v>2458</v>
+      </c>
+      <c r="AJ213" t="n">
+        <v>485</v>
+      </c>
+      <c r="AK213" t="n">
+        <v>88</v>
+      </c>
+      <c r="AL213" t="n">
+        <v>187</v>
+      </c>
+      <c r="AM213" t="n">
+        <v>0.9136</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="n">
+        <v>212</v>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>resnet34 baseline kfold | fold 3/5</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>resnet34</t>
+        </is>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>ImageNet</t>
+        </is>
+      </c>
+      <c r="F214" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G214" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H214" t="n">
+        <v>12494</v>
+      </c>
+      <c r="I214" t="n">
+        <v>70</v>
+      </c>
+      <c r="J214" t="n">
+        <v>10</v>
+      </c>
+      <c r="K214" t="n">
+        <v>20</v>
+      </c>
+      <c r="L214" t="n">
+        <v>2200</v>
+      </c>
+      <c r="M214" t="n">
+        <v>2421</v>
+      </c>
+      <c r="N214" t="n">
+        <v>807</v>
+      </c>
+      <c r="O214" t="n">
+        <v>807</v>
+      </c>
+      <c r="P214" t="n">
+        <v>807</v>
+      </c>
+      <c r="Q214" t="inlineStr">
+        <is>
+          <t>Per-subclass inverse frequency</t>
+        </is>
+      </c>
+      <c r="R214" t="inlineStr">
+        <is>
+          <t>AdamW</t>
+        </is>
+      </c>
+      <c r="S214" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="T214" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="U214" t="n">
+        <v>32</v>
+      </c>
+      <c r="V214" t="n">
+        <v>20</v>
+      </c>
+      <c r="W214" t="inlineStr">
+        <is>
+          <t>CosineAnnealingLR (T_max=20)</t>
+        </is>
+      </c>
+      <c r="X214" t="inlineStr">
+        <is>
+          <t>256x256</t>
+        </is>
+      </c>
+      <c r="Y214" t="inlineStr">
+        <is>
+          <t>HFlip, VFlip, Rotation(15°), ColorJitter(b=0.2,c=0.2), ImageNet norm</t>
+        </is>
+      </c>
+      <c r="Z214" t="n">
+        <v>0.9173</v>
+      </c>
+      <c r="AA214" t="n">
+        <v>0.7707000000000001</v>
+      </c>
+      <c r="AB214" t="n">
+        <v>0.7627</v>
+      </c>
+      <c r="AC214" t="n">
+        <v>0.7667</v>
+      </c>
+      <c r="AD214" t="n">
+        <v>0.9487</v>
+      </c>
+      <c r="AE214" t="n">
+        <v>0.9509</v>
+      </c>
+      <c r="AF214" t="n">
+        <v>0.9498</v>
+      </c>
+      <c r="AG214" t="n">
+        <v>0.8582</v>
+      </c>
+      <c r="AH214" t="n">
+        <v>0.9172</v>
+      </c>
+      <c r="AI214" t="n">
+        <v>2515</v>
+      </c>
+      <c r="AJ214" t="n">
+        <v>437</v>
+      </c>
+      <c r="AK214" t="n">
+        <v>136</v>
+      </c>
+      <c r="AL214" t="n">
+        <v>130</v>
+      </c>
+      <c r="AM214" t="n">
+        <v>0.9154</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="n">
+        <v>213</v>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>resnet34 baseline kfold | fold 4/5</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>resnet34</t>
+        </is>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>ImageNet</t>
+        </is>
+      </c>
+      <c r="F215" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G215" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H215" t="n">
+        <v>12494</v>
+      </c>
+      <c r="I215" t="n">
+        <v>70</v>
+      </c>
+      <c r="J215" t="n">
+        <v>10</v>
+      </c>
+      <c r="K215" t="n">
+        <v>20</v>
+      </c>
+      <c r="L215" t="n">
+        <v>2200</v>
+      </c>
+      <c r="M215" t="n">
+        <v>2421</v>
+      </c>
+      <c r="N215" t="n">
+        <v>807</v>
+      </c>
+      <c r="O215" t="n">
+        <v>807</v>
+      </c>
+      <c r="P215" t="n">
+        <v>807</v>
+      </c>
+      <c r="Q215" t="inlineStr">
+        <is>
+          <t>Per-subclass inverse frequency</t>
+        </is>
+      </c>
+      <c r="R215" t="inlineStr">
+        <is>
+          <t>AdamW</t>
+        </is>
+      </c>
+      <c r="S215" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="T215" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="U215" t="n">
+        <v>32</v>
+      </c>
+      <c r="V215" t="n">
+        <v>20</v>
+      </c>
+      <c r="W215" t="inlineStr">
+        <is>
+          <t>CosineAnnealingLR (T_max=20)</t>
+        </is>
+      </c>
+      <c r="X215" t="inlineStr">
+        <is>
+          <t>256x256</t>
+        </is>
+      </c>
+      <c r="Y215" t="inlineStr">
+        <is>
+          <t>HFlip, VFlip, Rotation(15°), ColorJitter(b=0.2,c=0.2), ImageNet norm</t>
+        </is>
+      </c>
+      <c r="Z215" t="n">
+        <v>0.9232</v>
+      </c>
+      <c r="AA215" t="n">
+        <v>0.789</v>
+      </c>
+      <c r="AB215" t="n">
+        <v>0.7766</v>
+      </c>
+      <c r="AC215" t="n">
+        <v>0.7828000000000001</v>
+      </c>
+      <c r="AD215" t="n">
+        <v>0.9518</v>
+      </c>
+      <c r="AE215" t="n">
+        <v>0.955</v>
+      </c>
+      <c r="AF215" t="n">
+        <v>0.9534</v>
+      </c>
+      <c r="AG215" t="n">
+        <v>0.8681</v>
+      </c>
+      <c r="AH215" t="n">
+        <v>0.923</v>
+      </c>
+      <c r="AI215" t="n">
+        <v>2526</v>
+      </c>
+      <c r="AJ215" t="n">
+        <v>445</v>
+      </c>
+      <c r="AK215" t="n">
+        <v>128</v>
+      </c>
+      <c r="AL215" t="n">
+        <v>119</v>
+      </c>
+      <c r="AM215" t="n">
+        <v>0.926</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="n">
+        <v>214</v>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>resnet34 baseline kfold | fold 5/5</t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>resnet34</t>
+        </is>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>ImageNet</t>
+        </is>
+      </c>
+      <c r="F216" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G216" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H216" t="n">
+        <v>12494</v>
+      </c>
+      <c r="I216" t="n">
+        <v>70</v>
+      </c>
+      <c r="J216" t="n">
+        <v>10</v>
+      </c>
+      <c r="K216" t="n">
+        <v>20</v>
+      </c>
+      <c r="L216" t="n">
+        <v>2200</v>
+      </c>
+      <c r="M216" t="n">
+        <v>2421</v>
+      </c>
+      <c r="N216" t="n">
+        <v>807</v>
+      </c>
+      <c r="O216" t="n">
+        <v>807</v>
+      </c>
+      <c r="P216" t="n">
+        <v>807</v>
+      </c>
+      <c r="Q216" t="inlineStr">
+        <is>
+          <t>Per-subclass inverse frequency</t>
+        </is>
+      </c>
+      <c r="R216" t="inlineStr">
+        <is>
+          <t>AdamW</t>
+        </is>
+      </c>
+      <c r="S216" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="T216" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="U216" t="n">
+        <v>32</v>
+      </c>
+      <c r="V216" t="n">
+        <v>20</v>
+      </c>
+      <c r="W216" t="inlineStr">
+        <is>
+          <t>CosineAnnealingLR (T_max=20)</t>
+        </is>
+      </c>
+      <c r="X216" t="inlineStr">
+        <is>
+          <t>256x256</t>
+        </is>
+      </c>
+      <c r="Y216" t="inlineStr">
+        <is>
+          <t>HFlip, VFlip, Rotation(15°), ColorJitter(b=0.2,c=0.2), ImageNet norm</t>
+        </is>
+      </c>
+      <c r="Z216" t="n">
+        <v>0.9173</v>
+      </c>
+      <c r="AA216" t="n">
+        <v>0.7433</v>
+      </c>
+      <c r="AB216" t="n">
+        <v>0.8185</v>
+      </c>
+      <c r="AC216" t="n">
+        <v>0.7791</v>
+      </c>
+      <c r="AD216" t="n">
+        <v>0.9598</v>
+      </c>
+      <c r="AE216" t="n">
+        <v>0.9388</v>
+      </c>
+      <c r="AF216" t="n">
+        <v>0.9492</v>
+      </c>
+      <c r="AG216" t="n">
+        <v>0.8641</v>
+      </c>
+      <c r="AH216" t="n">
+        <v>0.9189000000000001</v>
+      </c>
+      <c r="AI216" t="n">
+        <v>2483</v>
+      </c>
+      <c r="AJ216" t="n">
+        <v>469</v>
+      </c>
+      <c r="AK216" t="n">
+        <v>104</v>
+      </c>
+      <c r="AL216" t="n">
+        <v>162</v>
+      </c>
+      <c r="AM216" t="n">
+        <v>0.9192</v>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="n">
+        <v>215</v>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>resnet18</t>
+        </is>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>resnet18</t>
+        </is>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>ImageNet</t>
+        </is>
+      </c>
+      <c r="F217" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G217" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H217" t="inlineStr">
+        <is>
+          <t>RBC Count</t>
+        </is>
+      </c>
+      <c r="I217" t="n">
+        <v>70</v>
+      </c>
+      <c r="J217" t="n">
+        <v>10</v>
+      </c>
+      <c r="K217" t="n">
+        <v>20</v>
+      </c>
+      <c r="L217" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M217" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N217" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O217" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P217" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q217" t="inlineStr">
+        <is>
+          <t>Natural distribution</t>
+        </is>
+      </c>
+      <c r="R217" t="inlineStr">
+        <is>
+          <t>AdamW</t>
+        </is>
+      </c>
+      <c r="S217" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="T217" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="U217" t="n">
+        <v>32</v>
+      </c>
+      <c r="V217" t="n">
+        <v>20</v>
+      </c>
+      <c r="W217" t="inlineStr">
+        <is>
+          <t>CosineAnnealingLR (T_max=20)</t>
+        </is>
+      </c>
+      <c r="X217" t="inlineStr">
+        <is>
+          <t>256x256</t>
+        </is>
+      </c>
+      <c r="Y217" t="inlineStr">
+        <is>
+          <t>HFlip, VFlip, Rotation(15°), ColorJitter(b=0.2,c=0.2), ImageNet norm</t>
+        </is>
+      </c>
+      <c r="Z217" t="n">
+        <v>0.9676</v>
+      </c>
+      <c r="AA217" t="n">
+        <v>0.997</v>
+      </c>
+      <c r="AB217" t="n">
+        <v>0.9891</v>
+      </c>
+      <c r="AC217" t="n">
+        <v>0.9931</v>
+      </c>
+      <c r="AD217" t="n">
+        <v>0.8264</v>
+      </c>
+      <c r="AE217" t="n">
+        <v>0.9091</v>
+      </c>
+      <c r="AF217" t="n">
+        <v>0.8658</v>
+      </c>
+      <c r="AG217" t="n">
+        <v>0.8663</v>
+      </c>
+      <c r="AH217" t="n">
+        <v>0.9679</v>
+      </c>
+      <c r="AI217" t="n">
+        <v>0.9668</v>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="n">
+        <v>216</v>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>resnet34</t>
+        </is>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>resnet34</t>
+        </is>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>ImageNet</t>
+        </is>
+      </c>
+      <c r="F218" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G218" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H218" t="inlineStr">
+        <is>
+          <t>RBC Count</t>
+        </is>
+      </c>
+      <c r="I218" t="n">
+        <v>70</v>
+      </c>
+      <c r="J218" t="n">
+        <v>10</v>
+      </c>
+      <c r="K218" t="n">
+        <v>20</v>
+      </c>
+      <c r="L218" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M218" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N218" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O218" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P218" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q218" t="inlineStr">
+        <is>
+          <t>Natural distribution</t>
+        </is>
+      </c>
+      <c r="R218" t="inlineStr">
+        <is>
+          <t>AdamW</t>
+        </is>
+      </c>
+      <c r="S218" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="T218" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="U218" t="n">
+        <v>32</v>
+      </c>
+      <c r="V218" t="n">
+        <v>20</v>
+      </c>
+      <c r="W218" t="inlineStr">
+        <is>
+          <t>CosineAnnealingLR (T_max=20)</t>
+        </is>
+      </c>
+      <c r="X218" t="inlineStr">
+        <is>
+          <t>256x256</t>
+        </is>
+      </c>
+      <c r="Y218" t="inlineStr">
+        <is>
+          <t>HFlip, VFlip, Rotation(15°), ColorJitter(b=0.2,c=0.2), ImageNet norm</t>
+        </is>
+      </c>
+      <c r="Z218" t="n">
+        <v>0.9776</v>
+      </c>
+      <c r="AA218" t="n">
+        <v>0.997</v>
+      </c>
+      <c r="AB218" t="n">
+        <v>0.9941</v>
+      </c>
+      <c r="AC218" t="n">
+        <v>0.9955000000000001</v>
+      </c>
+      <c r="AD218" t="n">
+        <v>0.8974</v>
+      </c>
+      <c r="AE218" t="n">
+        <v>0.9545</v>
+      </c>
+      <c r="AF218" t="n">
+        <v>0.9251</v>
+      </c>
+      <c r="AG218" t="n">
+        <v>0.8932</v>
+      </c>
+      <c r="AH218" t="n">
+        <v>0.9775</v>
+      </c>
+      <c r="AI218" t="n">
+        <v>0.9751</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="n">
+        <v>217</v>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>resnet50</t>
+        </is>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>resnet50</t>
+        </is>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>ImageNet</t>
+        </is>
+      </c>
+      <c r="F219" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G219" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H219" t="inlineStr">
+        <is>
+          <t>RBC Count</t>
+        </is>
+      </c>
+      <c r="I219" t="n">
+        <v>70</v>
+      </c>
+      <c r="J219" t="n">
+        <v>10</v>
+      </c>
+      <c r="K219" t="n">
+        <v>20</v>
+      </c>
+      <c r="L219" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M219" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N219" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O219" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P219" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q219" t="inlineStr">
+        <is>
+          <t>Natural distribution</t>
+        </is>
+      </c>
+      <c r="R219" t="inlineStr">
+        <is>
+          <t>AdamW</t>
+        </is>
+      </c>
+      <c r="S219" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="T219" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="U219" t="n">
+        <v>32</v>
+      </c>
+      <c r="V219" t="n">
+        <v>20</v>
+      </c>
+      <c r="W219" t="inlineStr">
+        <is>
+          <t>CosineAnnealingLR (T_max=20)</t>
+        </is>
+      </c>
+      <c r="X219" t="inlineStr">
+        <is>
+          <t>256x256</t>
+        </is>
+      </c>
+      <c r="Y219" t="inlineStr">
+        <is>
+          <t>HFlip, VFlip, Rotation(15°), ColorJitter(b=0.2,c=0.2), ImageNet norm</t>
+        </is>
+      </c>
+      <c r="Z219" t="n">
+        <v>0.9734</v>
+      </c>
+      <c r="AA219" t="n">
+        <v>0.995</v>
+      </c>
+      <c r="AB219" t="n">
+        <v>0.9931</v>
+      </c>
+      <c r="AC219" t="n">
+        <v>0.9941</v>
+      </c>
+      <c r="AD219" t="n">
+        <v>0.8718</v>
+      </c>
+      <c r="AE219" t="n">
+        <v>0.9273</v>
+      </c>
+      <c r="AF219" t="n">
+        <v>0.8987000000000001</v>
+      </c>
+      <c r="AG219" t="n">
+        <v>0.883</v>
+      </c>
+      <c r="AH219" t="n">
+        <v>0.9733000000000001</v>
+      </c>
+      <c r="AI219" t="n">
+        <v>0.9718</v>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="n">
+        <v>218</v>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>resnet101</t>
+        </is>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>resnet101</t>
+        </is>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>ImageNet</t>
+        </is>
+      </c>
+      <c r="F220" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G220" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H220" t="inlineStr">
+        <is>
+          <t>RBC Count</t>
+        </is>
+      </c>
+      <c r="I220" t="n">
+        <v>70</v>
+      </c>
+      <c r="J220" t="n">
+        <v>10</v>
+      </c>
+      <c r="K220" t="n">
+        <v>20</v>
+      </c>
+      <c r="L220" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M220" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N220" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O220" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P220" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q220" t="inlineStr">
+        <is>
+          <t>Natural distribution</t>
+        </is>
+      </c>
+      <c r="R220" t="inlineStr">
+        <is>
+          <t>AdamW</t>
+        </is>
+      </c>
+      <c r="S220" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="T220" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="U220" t="n">
+        <v>32</v>
+      </c>
+      <c r="V220" t="n">
+        <v>20</v>
+      </c>
+      <c r="W220" t="inlineStr">
+        <is>
+          <t>CosineAnnealingLR (T_max=20)</t>
+        </is>
+      </c>
+      <c r="X220" t="inlineStr">
+        <is>
+          <t>256x256</t>
+        </is>
+      </c>
+      <c r="Y220" t="inlineStr">
+        <is>
+          <t>HFlip, VFlip, Rotation(15°), ColorJitter(b=0.2,c=0.2), ImageNet norm</t>
+        </is>
+      </c>
+      <c r="Z220" t="n">
+        <v>0.9776</v>
+      </c>
+      <c r="AA220" t="n">
+        <v>0.997</v>
+      </c>
+      <c r="AB220" t="n">
+        <v>0.9901</v>
+      </c>
+      <c r="AC220" t="n">
+        <v>0.9936</v>
+      </c>
+      <c r="AD220" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="AE220" t="n">
+        <v>0.9545</v>
+      </c>
+      <c r="AF220" t="n">
+        <v>0.913</v>
+      </c>
+      <c r="AG220" t="n">
+        <v>0.9124</v>
+      </c>
+      <c r="AH220" t="n">
+        <v>0.9776</v>
+      </c>
+      <c r="AI220" t="n">
+        <v>0.9801</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="n">
+        <v>219</v>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>resnet152</t>
+        </is>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>resnet152</t>
+        </is>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>ImageNet</t>
+        </is>
+      </c>
+      <c r="F221" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G221" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H221" t="inlineStr">
+        <is>
+          <t>RBC Count</t>
+        </is>
+      </c>
+      <c r="I221" t="n">
+        <v>70</v>
+      </c>
+      <c r="J221" t="n">
+        <v>10</v>
+      </c>
+      <c r="K221" t="n">
+        <v>20</v>
+      </c>
+      <c r="L221" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M221" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N221" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O221" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P221" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q221" t="inlineStr">
+        <is>
+          <t>Natural distribution</t>
+        </is>
+      </c>
+      <c r="R221" t="inlineStr">
+        <is>
+          <t>AdamW</t>
+        </is>
+      </c>
+      <c r="S221" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="T221" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="U221" t="n">
+        <v>32</v>
+      </c>
+      <c r="V221" t="n">
+        <v>20</v>
+      </c>
+      <c r="W221" t="inlineStr">
+        <is>
+          <t>CosineAnnealingLR (T_max=20)</t>
+        </is>
+      </c>
+      <c r="X221" t="inlineStr">
+        <is>
+          <t>256x256</t>
+        </is>
+      </c>
+      <c r="Y221" t="inlineStr">
+        <is>
+          <t>HFlip, VFlip, Rotation(15°), ColorJitter(b=0.2,c=0.2), ImageNet norm</t>
+        </is>
+      </c>
+      <c r="Z221" t="n">
+        <v>0.9792</v>
+      </c>
+      <c r="AA221" t="n">
+        <v>0.997</v>
+      </c>
+      <c r="AB221" t="n">
+        <v>0.996</v>
+      </c>
+      <c r="AC221" t="n">
+        <v>0.9965000000000001</v>
+      </c>
+      <c r="AD221" t="n">
+        <v>0.9211</v>
+      </c>
+      <c r="AE221" t="n">
+        <v>0.9545</v>
+      </c>
+      <c r="AF221" t="n">
+        <v>0.9375</v>
+      </c>
+      <c r="AG221" t="n">
+        <v>0.893</v>
+      </c>
+      <c r="AH221" t="n">
+        <v>0.9789</v>
+      </c>
+      <c r="AI221" t="n">
+        <v>0.9734</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="n">
+        <v>220</v>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>efficientnet_b0</t>
+        </is>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>efficientnet_b0</t>
+        </is>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>ImageNet</t>
+        </is>
+      </c>
+      <c r="F222" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G222" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H222" t="inlineStr">
+        <is>
+          <t>RBC Count</t>
+        </is>
+      </c>
+      <c r="I222" t="n">
+        <v>70</v>
+      </c>
+      <c r="J222" t="n">
+        <v>10</v>
+      </c>
+      <c r="K222" t="n">
+        <v>20</v>
+      </c>
+      <c r="L222" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M222" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N222" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O222" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P222" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q222" t="inlineStr">
+        <is>
+          <t>Natural distribution</t>
+        </is>
+      </c>
+      <c r="R222" t="inlineStr">
+        <is>
+          <t>AdamW</t>
+        </is>
+      </c>
+      <c r="S222" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="T222" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="U222" t="n">
+        <v>32</v>
+      </c>
+      <c r="V222" t="n">
+        <v>20</v>
+      </c>
+      <c r="W222" t="inlineStr">
+        <is>
+          <t>CosineAnnealingLR (T_max=20)</t>
+        </is>
+      </c>
+      <c r="X222" t="inlineStr">
+        <is>
+          <t>256x256</t>
+        </is>
+      </c>
+      <c r="Y222" t="inlineStr">
+        <is>
+          <t>HFlip, VFlip, Rotation(15°), ColorJitter(b=0.2,c=0.2), ImageNet norm</t>
+        </is>
+      </c>
+      <c r="Z222" t="n">
+        <v>0.9692</v>
+      </c>
+      <c r="AA222" t="n">
+        <v>0.995</v>
+      </c>
+      <c r="AB222" t="n">
+        <v>0.9911</v>
+      </c>
+      <c r="AC222" t="n">
+        <v>0.9931</v>
+      </c>
+      <c r="AD222" t="n">
+        <v>0.8475</v>
+      </c>
+      <c r="AE222" t="n">
+        <v>0.9091</v>
+      </c>
+      <c r="AF222" t="n">
+        <v>0.8772</v>
+      </c>
+      <c r="AG222" t="n">
+        <v>0.8698</v>
+      </c>
+      <c r="AH222" t="n">
+        <v>0.9689</v>
+      </c>
+      <c r="AI222" t="n">
+        <v>0.9550999999999999</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="n">
+        <v>221</v>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>efficientnet_b1</t>
+        </is>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>efficientnet_b1</t>
+        </is>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>ImageNet</t>
+        </is>
+      </c>
+      <c r="F223" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G223" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H223" t="inlineStr">
+        <is>
+          <t>RBC Count</t>
+        </is>
+      </c>
+      <c r="I223" t="n">
+        <v>70</v>
+      </c>
+      <c r="J223" t="n">
+        <v>10</v>
+      </c>
+      <c r="K223" t="n">
+        <v>20</v>
+      </c>
+      <c r="L223" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M223" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N223" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O223" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P223" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q223" t="inlineStr">
+        <is>
+          <t>Natural distribution</t>
+        </is>
+      </c>
+      <c r="R223" t="inlineStr">
+        <is>
+          <t>AdamW</t>
+        </is>
+      </c>
+      <c r="S223" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="T223" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="U223" t="n">
+        <v>32</v>
+      </c>
+      <c r="V223" t="n">
+        <v>20</v>
+      </c>
+      <c r="W223" t="inlineStr">
+        <is>
+          <t>CosineAnnealingLR (T_max=20)</t>
+        </is>
+      </c>
+      <c r="X223" t="inlineStr">
+        <is>
+          <t>256x256</t>
+        </is>
+      </c>
+      <c r="Y223" t="inlineStr">
+        <is>
+          <t>HFlip, VFlip, Rotation(15°), ColorJitter(b=0.2,c=0.2), ImageNet norm</t>
+        </is>
+      </c>
+      <c r="Z223" t="n">
+        <v>0.9543</v>
+      </c>
+      <c r="AA223" t="n">
+        <v>0.993</v>
+      </c>
+      <c r="AB223" t="n">
+        <v>0.9832</v>
+      </c>
+      <c r="AC223" t="n">
+        <v>0.9881</v>
+      </c>
+      <c r="AD223" t="n">
+        <v>0.7805</v>
+      </c>
+      <c r="AE223" t="n">
+        <v>0.8727</v>
+      </c>
+      <c r="AF223" t="n">
+        <v>0.824</v>
+      </c>
+      <c r="AG223" t="n">
+        <v>0.8144</v>
+      </c>
+      <c r="AH223" t="n">
+        <v>0.9546</v>
+      </c>
+      <c r="AI223" t="n">
+        <v>0.9419</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="n">
+        <v>222</v>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>efficientnet_b4</t>
+        </is>
+      </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>efficientnet_b4</t>
+        </is>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>ImageNet</t>
+        </is>
+      </c>
+      <c r="F224" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G224" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H224" t="inlineStr">
+        <is>
+          <t>RBC Count</t>
+        </is>
+      </c>
+      <c r="I224" t="n">
+        <v>70</v>
+      </c>
+      <c r="J224" t="n">
+        <v>10</v>
+      </c>
+      <c r="K224" t="n">
+        <v>20</v>
+      </c>
+      <c r="L224" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M224" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N224" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O224" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P224" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q224" t="inlineStr">
+        <is>
+          <t>Natural distribution</t>
+        </is>
+      </c>
+      <c r="R224" t="inlineStr">
+        <is>
+          <t>AdamW</t>
+        </is>
+      </c>
+      <c r="S224" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="T224" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="U224" t="n">
+        <v>32</v>
+      </c>
+      <c r="V224" t="n">
+        <v>20</v>
+      </c>
+      <c r="W224" t="inlineStr">
+        <is>
+          <t>CosineAnnealingLR (T_max=20)</t>
+        </is>
+      </c>
+      <c r="X224" t="inlineStr">
+        <is>
+          <t>256x256</t>
+        </is>
+      </c>
+      <c r="Y224" t="inlineStr">
+        <is>
+          <t>HFlip, VFlip, Rotation(15°), ColorJitter(b=0.2,c=0.2), ImageNet norm</t>
+        </is>
+      </c>
+      <c r="Z224" t="n">
+        <v>0.9601</v>
+      </c>
+      <c r="AA224" t="n">
+        <v>0.995</v>
+      </c>
+      <c r="AB224" t="n">
+        <v>0.9901</v>
+      </c>
+      <c r="AC224" t="n">
+        <v>0.9926</v>
+      </c>
+      <c r="AD224" t="n">
+        <v>0.8115</v>
+      </c>
+      <c r="AE224" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AF224" t="n">
+        <v>0.8534</v>
+      </c>
+      <c r="AG224" t="n">
+        <v>0.8163</v>
+      </c>
+      <c r="AH224" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="AI224" t="n">
+        <v>0.9485</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="R1:Y1"/>

</xml_diff>

<commit_message>
Attempted to train a custom model for segmentation
</commit_message>
<xml_diff>
--- a/experiment_log.xlsx
+++ b/experiment_log.xlsx
@@ -599,7 +599,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR224"/>
+  <dimension ref="A1:AR227"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -31996,6 +31996,423 @@
         <v>0.9485</v>
       </c>
     </row>
+    <row r="225">
+      <c r="A225" t="n">
+        <v>223</v>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>convnext_tiny</t>
+        </is>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>convnext_tiny</t>
+        </is>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>ImageNet</t>
+        </is>
+      </c>
+      <c r="F225" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G225" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H225" t="inlineStr">
+        <is>
+          <t>RBC Count</t>
+        </is>
+      </c>
+      <c r="I225" t="n">
+        <v>70</v>
+      </c>
+      <c r="J225" t="n">
+        <v>10</v>
+      </c>
+      <c r="K225" t="n">
+        <v>20</v>
+      </c>
+      <c r="L225" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M225" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N225" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O225" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P225" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q225" t="inlineStr">
+        <is>
+          <t>Natural distribution</t>
+        </is>
+      </c>
+      <c r="R225" t="inlineStr">
+        <is>
+          <t>AdamW</t>
+        </is>
+      </c>
+      <c r="S225" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="T225" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="U225" t="n">
+        <v>32</v>
+      </c>
+      <c r="V225" t="n">
+        <v>20</v>
+      </c>
+      <c r="W225" t="inlineStr">
+        <is>
+          <t>CosineAnnealingLR (T_max=20)</t>
+        </is>
+      </c>
+      <c r="X225" t="inlineStr">
+        <is>
+          <t>256x256</t>
+        </is>
+      </c>
+      <c r="Y225" t="inlineStr">
+        <is>
+          <t>HFlip, VFlip, Rotation(15°), ColorJitter(b=0.2,c=0.2), ImageNet norm</t>
+        </is>
+      </c>
+      <c r="Z225" t="n">
+        <v>0.9767</v>
+      </c>
+      <c r="AA225" t="n">
+        <v>0.996</v>
+      </c>
+      <c r="AB225" t="n">
+        <v>0.9941</v>
+      </c>
+      <c r="AC225" t="n">
+        <v>0.9951</v>
+      </c>
+      <c r="AD225" t="n">
+        <v>0.9196</v>
+      </c>
+      <c r="AE225" t="n">
+        <v>0.9364</v>
+      </c>
+      <c r="AF225" t="n">
+        <v>0.9278999999999999</v>
+      </c>
+      <c r="AG225" t="n">
+        <v>0.8891</v>
+      </c>
+      <c r="AH225" t="n">
+        <v>0.9766</v>
+      </c>
+      <c r="AI225" t="n">
+        <v>0.9784</v>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="n">
+        <v>224</v>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>convnext_base</t>
+        </is>
+      </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>convnext_base</t>
+        </is>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>ImageNet</t>
+        </is>
+      </c>
+      <c r="F226" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G226" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H226" t="inlineStr">
+        <is>
+          <t>RBC Count</t>
+        </is>
+      </c>
+      <c r="I226" t="n">
+        <v>70</v>
+      </c>
+      <c r="J226" t="n">
+        <v>10</v>
+      </c>
+      <c r="K226" t="n">
+        <v>20</v>
+      </c>
+      <c r="L226" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M226" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N226" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O226" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P226" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q226" t="inlineStr">
+        <is>
+          <t>Natural distribution</t>
+        </is>
+      </c>
+      <c r="R226" t="inlineStr">
+        <is>
+          <t>AdamW</t>
+        </is>
+      </c>
+      <c r="S226" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="T226" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="U226" t="n">
+        <v>32</v>
+      </c>
+      <c r="V226" t="n">
+        <v>20</v>
+      </c>
+      <c r="W226" t="inlineStr">
+        <is>
+          <t>CosineAnnealingLR (T_max=20)</t>
+        </is>
+      </c>
+      <c r="X226" t="inlineStr">
+        <is>
+          <t>256x256</t>
+        </is>
+      </c>
+      <c r="Y226" t="inlineStr">
+        <is>
+          <t>HFlip, VFlip, Rotation(15°), ColorJitter(b=0.2,c=0.2), ImageNet norm</t>
+        </is>
+      </c>
+      <c r="Z226" t="n">
+        <v>0.9825</v>
+      </c>
+      <c r="AA226" t="n">
+        <v>0.997</v>
+      </c>
+      <c r="AB226" t="n">
+        <v>0.9921</v>
+      </c>
+      <c r="AC226" t="n">
+        <v>0.9946</v>
+      </c>
+      <c r="AD226" t="n">
+        <v>0.9137999999999999</v>
+      </c>
+      <c r="AE226" t="n">
+        <v>0.9636</v>
+      </c>
+      <c r="AF226" t="n">
+        <v>0.9381</v>
+      </c>
+      <c r="AG226" t="n">
+        <v>0.9306</v>
+      </c>
+      <c r="AH226" t="n">
+        <v>0.9826</v>
+      </c>
+      <c r="AI226" t="n">
+        <v>0.9767</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="n">
+        <v>225</v>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>vit_b16</t>
+        </is>
+      </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>vit_b16</t>
+        </is>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>ImageNet</t>
+        </is>
+      </c>
+      <c r="F227" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G227" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H227" t="inlineStr">
+        <is>
+          <t>RBC Count</t>
+        </is>
+      </c>
+      <c r="I227" t="n">
+        <v>70</v>
+      </c>
+      <c r="J227" t="n">
+        <v>10</v>
+      </c>
+      <c r="K227" t="n">
+        <v>20</v>
+      </c>
+      <c r="L227" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M227" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N227" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O227" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P227" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q227" t="inlineStr">
+        <is>
+          <t>Natural distribution</t>
+        </is>
+      </c>
+      <c r="R227" t="inlineStr">
+        <is>
+          <t>AdamW</t>
+        </is>
+      </c>
+      <c r="S227" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="T227" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="U227" t="n">
+        <v>32</v>
+      </c>
+      <c r="V227" t="n">
+        <v>20</v>
+      </c>
+      <c r="W227" t="inlineStr">
+        <is>
+          <t>CosineAnnealingLR (T_max=20)</t>
+        </is>
+      </c>
+      <c r="X227" t="inlineStr">
+        <is>
+          <t>256x256</t>
+        </is>
+      </c>
+      <c r="Y227" t="inlineStr">
+        <is>
+          <t>HFlip, VFlip, Rotation(15°), ColorJitter(b=0.2,c=0.2), ImageNet norm</t>
+        </is>
+      </c>
+      <c r="Z227" t="n">
+        <v>0.9684</v>
+      </c>
+      <c r="AA227" t="n">
+        <v>0.9941</v>
+      </c>
+      <c r="AB227" t="n">
+        <v>0.996</v>
+      </c>
+      <c r="AC227" t="n">
+        <v>0.9951</v>
+      </c>
+      <c r="AD227" t="n">
+        <v>0.8632</v>
+      </c>
+      <c r="AE227" t="n">
+        <v>0.9182</v>
+      </c>
+      <c r="AF227" t="n">
+        <v>0.8899</v>
+      </c>
+      <c r="AG227" t="n">
+        <v>0.8413</v>
+      </c>
+      <c r="AH227" t="n">
+        <v>0.9675</v>
+      </c>
+      <c r="AI227" t="n">
+        <v>0.9718</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="R1:Y1"/>

</xml_diff>